<commit_message>
Before adding web crawler
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/db_code lookups/Business Category and Search.xlsx
+++ b/assets/db_code lookups/Business Category and Search.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ac97c493c1628ead/Documents/Personal Stuff/Code Projects/Avtopia/Business Search/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jared\source\repos\data_sync_desktop\assets\db_code lookups\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DC2B1247-4DBE-4868-9F1C-9151718963C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EC1C613-0C48-442A-AF1A-FC8B7EA119C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F6BDE4B6-EF96-429D-83BC-A8CA702EE26E}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F6BDE4B6-EF96-429D-83BC-A8CA702EE26E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$139</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -6298,6 +6301,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I139" xr:uid="{F3E636FB-4402-4645-9A44-82EBF6022327}"/>
   <conditionalFormatting sqref="D145:D1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Commit before importing from FAA document
</commit_message>
<xml_diff>
--- a/assets/db_code lookups/Business Category and Search.xlsx
+++ b/assets/db_code lookups/Business Category and Search.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jared\source\repos\data_sync_desktop\assets\db_code lookups\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EC1C613-0C48-442A-AF1A-FC8B7EA119C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{363760AF-45C9-4EAA-B5ED-174C56455814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F6BDE4B6-EF96-429D-83BC-A8CA702EE26E}"/>
   </bookViews>
@@ -269,9 +269,6 @@
     <t>International Airline (CFR 121)</t>
   </si>
   <si>
-    <t>MAJ121</t>
-  </si>
-  <si>
     <t>airline | international | major airline | 121| big airline | air carrier | major carrier</t>
   </si>
   <si>
@@ -1781,6 +1778,9 @@
   </si>
   <si>
     <t xml:space="preserve">Maintenance </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -3143,7 +3143,7 @@
         <v>75</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>76</v>
+        <v>569</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>0</v>
@@ -3155,21 +3155,21 @@
         <v>7</v>
       </c>
       <c r="H18" s="12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B19" s="30" t="s">
         <v>69</v>
       </c>
       <c r="C19" s="33" t="s">
+        <v>78</v>
+      </c>
+      <c r="D19" s="34" t="s">
         <v>79</v>
-      </c>
-      <c r="D19" s="34" t="s">
-        <v>80</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>0</v>
@@ -3181,21 +3181,21 @@
         <v>6</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="35" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B20" s="36" t="s">
         <v>69</v>
       </c>
       <c r="C20" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="D20" s="38" t="s">
         <v>83</v>
-      </c>
-      <c r="D20" s="38" t="s">
-        <v>84</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>0</v>
@@ -3207,12 +3207,12 @@
         <v>7</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="35" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B21" s="39" t="s">
         <v>69</v>
@@ -3238,94 +3238,94 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="42" t="s">
         <v>87</v>
       </c>
-      <c r="B22" s="42" t="s">
+      <c r="C22" s="43" t="s">
         <v>88</v>
       </c>
-      <c r="C22" s="43" t="s">
+      <c r="D22" s="44" t="s">
         <v>89</v>
       </c>
-      <c r="D22" s="44" t="s">
+      <c r="E22" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F22" s="45" t="s">
         <v>90</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F22" s="45" t="s">
-        <v>91</v>
       </c>
       <c r="G22" s="11">
         <v>7</v>
       </c>
       <c r="H22" s="12" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="C23" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="B23" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="C23" s="18" t="s">
+      <c r="D23" s="28" t="s">
         <v>94</v>
       </c>
-      <c r="D23" s="28" t="s">
-        <v>95</v>
-      </c>
       <c r="E23" s="2" t="s">
         <v>0</v>
       </c>
       <c r="F23" s="46" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G23" s="15">
         <v>8</v>
       </c>
       <c r="H23" s="16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="C24" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="B24" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="C24" s="18" t="s">
+      <c r="D24" s="28" t="s">
         <v>98</v>
       </c>
-      <c r="D24" s="28" t="s">
-        <v>99</v>
-      </c>
       <c r="E24" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F24" s="45" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G24" s="11">
         <v>5</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="B25" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="C25" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="B25" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="C25" s="18" t="s">
+      <c r="D25" s="28" t="s">
         <v>102</v>
-      </c>
-      <c r="D25" s="28" t="s">
-        <v>103</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>0</v>
@@ -3337,15 +3337,15 @@
         <v>8</v>
       </c>
       <c r="H25" s="12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C26" s="18" t="s">
         <v>42</v>
@@ -3368,218 +3368,218 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B27" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="B27" s="30" t="s">
+      <c r="C27" s="31" t="s">
         <v>107</v>
       </c>
-      <c r="C27" s="31" t="s">
+      <c r="D27" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="E27" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F27" s="47" t="s">
         <v>109</v>
-      </c>
-      <c r="E27" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F27" s="47" t="s">
-        <v>110</v>
       </c>
       <c r="G27" s="11">
         <v>10</v>
       </c>
       <c r="H27" s="12" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="B28" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="C28" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="B28" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="C28" s="31" t="s">
+      <c r="D28" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="D28" s="9" t="s">
-        <v>114</v>
-      </c>
       <c r="E28" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F28" s="47" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G28" s="11">
         <v>10</v>
       </c>
       <c r="H28" s="12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="B29" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="C29" s="31" t="s">
         <v>116</v>
       </c>
-      <c r="B29" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="C29" s="31" t="s">
+      <c r="D29" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="D29" s="9" t="s">
-        <v>118</v>
-      </c>
       <c r="E29" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F29" s="47" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G29" s="11">
         <v>10</v>
       </c>
       <c r="H29" s="12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="B30" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="C30" s="31" t="s">
         <v>120</v>
       </c>
-      <c r="B30" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="C30" s="31" t="s">
+      <c r="D30" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="D30" s="9" t="s">
-        <v>122</v>
-      </c>
       <c r="E30" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F30" s="47" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G30" s="11">
         <v>3</v>
       </c>
       <c r="H30" s="12" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="B31" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="C31" s="31" t="s">
         <v>124</v>
       </c>
-      <c r="B31" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="C31" s="31" t="s">
+      <c r="D31" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="D31" s="9" t="s">
-        <v>126</v>
-      </c>
       <c r="E31" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F31" s="47" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G31" s="11">
         <v>8</v>
       </c>
       <c r="H31" s="12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B32" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="C32" s="31" t="s">
         <v>128</v>
       </c>
-      <c r="B32" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="C32" s="31" t="s">
+      <c r="D32" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="D32" s="9" t="s">
-        <v>130</v>
-      </c>
       <c r="E32" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F32" s="47" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G32" s="11">
         <v>3</v>
       </c>
       <c r="H32" s="12" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B33" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="C33" s="48" t="s">
         <v>132</v>
       </c>
-      <c r="B33" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="C33" s="48" t="s">
+      <c r="D33" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="D33" s="9" t="s">
+      <c r="E33" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F33" s="49" t="s">
         <v>134</v>
-      </c>
-      <c r="E33" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F33" s="49" t="s">
-        <v>135</v>
       </c>
       <c r="G33" s="11">
         <v>4</v>
       </c>
       <c r="H33" s="12" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="B34" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="C34" s="31" t="s">
         <v>137</v>
       </c>
-      <c r="B34" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="C34" s="31" t="s">
+      <c r="D34" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="D34" s="9" t="s">
-        <v>139</v>
-      </c>
       <c r="E34" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F34" s="49" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G34" s="11">
         <v>3</v>
       </c>
       <c r="H34" s="12" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B35" s="30" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C35" s="31" t="s">
         <v>42</v>
@@ -3602,629 +3602,629 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="B36" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="C36" s="50" t="s">
         <v>142</v>
       </c>
-      <c r="B36" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="C36" s="50" t="s">
+      <c r="D36" s="51" t="s">
         <v>143</v>
-      </c>
-      <c r="D36" s="51" t="s">
-        <v>144</v>
       </c>
       <c r="E36" s="10"/>
       <c r="F36" s="47" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G36" s="11">
         <v>3</v>
       </c>
       <c r="H36" s="12" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="B37" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="C37" s="50" t="s">
         <v>146</v>
       </c>
-      <c r="B37" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="C37" s="50" t="s">
+      <c r="D37" s="51" t="s">
         <v>147</v>
-      </c>
-      <c r="D37" s="51" t="s">
-        <v>148</v>
       </c>
       <c r="E37" s="10"/>
       <c r="F37" s="47" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G37" s="11">
         <v>4</v>
       </c>
       <c r="H37" s="52" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="B38" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="C38" s="50" t="s">
         <v>150</v>
       </c>
-      <c r="B38" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="C38" s="50" t="s">
+      <c r="D38" s="51" t="s">
         <v>151</v>
-      </c>
-      <c r="D38" s="51" t="s">
-        <v>152</v>
       </c>
       <c r="E38" s="10"/>
       <c r="F38" s="47" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G38" s="11">
         <v>6</v>
       </c>
       <c r="H38" s="12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="B39" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="C39" s="53" t="s">
         <v>154</v>
       </c>
-      <c r="B39" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="C39" s="53" t="s">
+      <c r="D39" s="54" t="s">
         <v>155</v>
-      </c>
-      <c r="D39" s="54" t="s">
-        <v>156</v>
       </c>
       <c r="E39" s="55"/>
       <c r="F39" s="47" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G39" s="56">
         <v>11</v>
       </c>
       <c r="H39" s="57" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="B40" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="B40" s="17" t="s">
+      <c r="C40" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="C40" s="18" t="s">
+      <c r="D40" s="28" t="s">
         <v>160</v>
       </c>
-      <c r="D40" s="28" t="s">
+      <c r="E40" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F40" s="58" t="s">
         <v>161</v>
-      </c>
-      <c r="E40" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F40" s="58" t="s">
-        <v>162</v>
       </c>
       <c r="G40" s="11">
         <v>9</v>
       </c>
       <c r="H40" s="12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="B41" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="C41" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="B41" s="17" t="s">
-        <v>159</v>
-      </c>
-      <c r="C41" s="18" t="s">
+      <c r="D41" s="28" t="s">
         <v>165</v>
       </c>
-      <c r="D41" s="28" t="s">
-        <v>166</v>
-      </c>
       <c r="E41" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F41" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G41" s="11">
         <v>12</v>
       </c>
       <c r="H41" s="12" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="B42" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="C42" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="B42" s="17" t="s">
-        <v>159</v>
-      </c>
-      <c r="C42" s="18" t="s">
+      <c r="D42" s="28" t="s">
         <v>169</v>
       </c>
-      <c r="D42" s="28" t="s">
-        <v>170</v>
-      </c>
       <c r="E42" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F42" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G42" s="11">
         <v>7</v>
       </c>
       <c r="H42" s="12" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="B43" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="C43" s="29" t="s">
         <v>172</v>
       </c>
-      <c r="B43" s="17" t="s">
-        <v>159</v>
-      </c>
-      <c r="C43" s="29" t="s">
+      <c r="D43" s="28" t="s">
         <v>173</v>
       </c>
-      <c r="D43" s="28" t="s">
-        <v>174</v>
-      </c>
       <c r="E43" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F43" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G43" s="11">
         <v>7</v>
       </c>
       <c r="H43" s="12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="B44" s="59" t="s">
+        <v>158</v>
+      </c>
+      <c r="C44" s="60" t="s">
         <v>176</v>
       </c>
-      <c r="B44" s="59" t="s">
-        <v>159</v>
-      </c>
-      <c r="C44" s="60" t="s">
+      <c r="D44" s="19" t="s">
         <v>177</v>
       </c>
-      <c r="D44" s="19" t="s">
-        <v>178</v>
-      </c>
       <c r="E44" s="2" t="s">
         <v>0</v>
       </c>
       <c r="F44" s="61" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G44" s="15">
         <v>5</v>
       </c>
       <c r="H44" s="16" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="B45" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="C45" s="60" t="s">
         <v>180</v>
       </c>
-      <c r="B45" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="C45" s="60" t="s">
+      <c r="D45" s="28" t="s">
         <v>181</v>
       </c>
-      <c r="D45" s="28" t="s">
-        <v>182</v>
-      </c>
       <c r="E45" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F45" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G45" s="11">
         <v>5</v>
       </c>
       <c r="H45" s="12" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="B46" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="C46" s="60" t="s">
         <v>184</v>
       </c>
-      <c r="B46" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="C46" s="60" t="s">
+      <c r="D46" s="28" t="s">
         <v>185</v>
       </c>
-      <c r="D46" s="28" t="s">
-        <v>186</v>
-      </c>
       <c r="E46" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F46" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G46" s="11">
         <v>2</v>
       </c>
       <c r="H46" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="B47" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="C47" s="60" t="s">
         <v>188</v>
       </c>
-      <c r="B47" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="C47" s="60" t="s">
+      <c r="D47" s="28" t="s">
         <v>189</v>
       </c>
-      <c r="D47" s="28" t="s">
-        <v>190</v>
-      </c>
       <c r="E47" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F47" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G47" s="11">
         <v>13</v>
       </c>
       <c r="H47" s="12" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="B48" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="C48" s="60" t="s">
         <v>192</v>
       </c>
-      <c r="B48" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="C48" s="60" t="s">
+      <c r="D48" s="28" t="s">
         <v>193</v>
       </c>
-      <c r="D48" s="28" t="s">
-        <v>194</v>
-      </c>
       <c r="E48" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F48" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G48" s="11">
         <v>4</v>
       </c>
       <c r="H48" s="12" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="B49" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="C49" s="60" t="s">
         <v>196</v>
       </c>
-      <c r="B49" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="C49" s="60" t="s">
+      <c r="D49" s="28" t="s">
         <v>197</v>
       </c>
-      <c r="D49" s="28" t="s">
-        <v>198</v>
-      </c>
       <c r="E49" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F49" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G49" s="11">
         <v>2</v>
       </c>
       <c r="H49" s="12" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="B50" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="C50" s="60" t="s">
         <v>200</v>
       </c>
-      <c r="B50" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="C50" s="60" t="s">
+      <c r="D50" s="28" t="s">
         <v>201</v>
       </c>
-      <c r="D50" s="28" t="s">
-        <v>202</v>
-      </c>
       <c r="E50" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F50" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G50" s="11">
         <v>2</v>
       </c>
       <c r="H50" s="12" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="B51" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="C51" s="60" t="s">
         <v>204</v>
       </c>
-      <c r="B51" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="C51" s="60" t="s">
+      <c r="D51" s="28" t="s">
         <v>205</v>
       </c>
-      <c r="D51" s="28" t="s">
-        <v>206</v>
-      </c>
       <c r="E51" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F51" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G51" s="11">
         <v>4</v>
       </c>
       <c r="H51" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B52" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="C52" s="60" t="s">
         <v>208</v>
       </c>
-      <c r="B52" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="C52" s="60" t="s">
+      <c r="D52" s="28" t="s">
         <v>209</v>
       </c>
-      <c r="D52" s="28" t="s">
-        <v>210</v>
-      </c>
       <c r="E52" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F52" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G52" s="11">
         <v>4</v>
       </c>
       <c r="H52" s="12" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="B53" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="C53" s="60" t="s">
         <v>212</v>
       </c>
-      <c r="B53" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="C53" s="60" t="s">
+      <c r="D53" s="28" t="s">
         <v>213</v>
       </c>
-      <c r="D53" s="28" t="s">
-        <v>214</v>
-      </c>
       <c r="E53" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F53" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G53" s="11">
         <v>3</v>
       </c>
       <c r="H53" s="12" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="B54" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="C54" s="60" t="s">
         <v>216</v>
       </c>
-      <c r="B54" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="C54" s="60" t="s">
+      <c r="D54" s="28" t="s">
         <v>217</v>
       </c>
-      <c r="D54" s="28" t="s">
-        <v>218</v>
-      </c>
       <c r="E54" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F54" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G54" s="11">
         <v>6</v>
       </c>
       <c r="H54" s="12" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="B55" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="C55" s="60" t="s">
         <v>220</v>
       </c>
-      <c r="B55" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="C55" s="60" t="s">
+      <c r="D55" s="28" t="s">
         <v>221</v>
       </c>
-      <c r="D55" s="28" t="s">
-        <v>222</v>
-      </c>
       <c r="E55" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F55" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G55" s="11">
         <v>4</v>
       </c>
       <c r="H55" s="12" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="B56" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="C56" s="60" t="s">
         <v>224</v>
       </c>
-      <c r="B56" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="C56" s="60" t="s">
+      <c r="D56" s="28" t="s">
         <v>225</v>
       </c>
-      <c r="D56" s="28" t="s">
-        <v>226</v>
-      </c>
       <c r="E56" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F56" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G56" s="11">
         <v>3</v>
       </c>
       <c r="H56" s="52" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="B57" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="C57" s="60" t="s">
         <v>228</v>
       </c>
-      <c r="B57" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="C57" s="60" t="s">
+      <c r="D57" s="28" t="s">
         <v>229</v>
       </c>
-      <c r="D57" s="28" t="s">
-        <v>230</v>
-      </c>
       <c r="E57" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F57" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G57" s="11">
         <v>3</v>
       </c>
       <c r="H57" s="12" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="B58" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="C58" s="60" t="s">
         <v>232</v>
       </c>
-      <c r="B58" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="C58" s="60" t="s">
+      <c r="D58" s="28" t="s">
         <v>233</v>
       </c>
-      <c r="D58" s="28" t="s">
-        <v>234</v>
-      </c>
       <c r="E58" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F58" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G58" s="11">
         <v>3</v>
       </c>
       <c r="H58" s="12" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="B59" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="C59" s="60" t="s">
         <v>236</v>
       </c>
-      <c r="B59" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="C59" s="60" t="s">
+      <c r="D59" s="28" t="s">
         <v>237</v>
       </c>
-      <c r="D59" s="28" t="s">
-        <v>238</v>
-      </c>
       <c r="E59" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F59" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G59" s="11">
         <v>2</v>
       </c>
       <c r="H59" s="57" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="B60" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="C60" s="62" t="s">
         <v>240</v>
-      </c>
-      <c r="B60" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="C60" s="62" t="s">
-        <v>241</v>
       </c>
       <c r="D60" s="63" t="s">
         <v>43</v>
@@ -4242,528 +4242,528 @@
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="B61" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="C61" s="65" t="s">
         <v>242</v>
       </c>
-      <c r="B61" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="C61" s="65" t="s">
+      <c r="D61" s="66" t="s">
         <v>243</v>
-      </c>
-      <c r="D61" s="66" t="s">
-        <v>244</v>
       </c>
       <c r="E61" s="67"/>
       <c r="F61" s="68" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G61" s="64">
         <v>4</v>
       </c>
       <c r="H61" s="52" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="B62" s="8" t="s">
         <v>246</v>
       </c>
-      <c r="B62" s="8" t="s">
+      <c r="C62" s="8" t="s">
         <v>247</v>
       </c>
-      <c r="C62" s="8" t="s">
+      <c r="D62" s="9" t="s">
         <v>248</v>
       </c>
-      <c r="D62" s="9" t="s">
+      <c r="E62" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F62" s="69" t="s">
         <v>249</v>
-      </c>
-      <c r="E62" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F62" s="69" t="s">
-        <v>250</v>
       </c>
       <c r="G62" s="11">
         <v>7</v>
       </c>
       <c r="H62" s="12" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="B63" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C63" s="8" t="s">
         <v>252</v>
       </c>
-      <c r="B63" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="C63" s="8" t="s">
+      <c r="D63" s="9" t="s">
         <v>253</v>
       </c>
-      <c r="D63" s="9" t="s">
-        <v>254</v>
-      </c>
       <c r="E63" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F63" s="69" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G63" s="11">
         <v>4</v>
       </c>
       <c r="H63" s="12" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C64" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="B64" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="C64" s="8" t="s">
+      <c r="D64" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="D64" s="9" t="s">
-        <v>258</v>
-      </c>
       <c r="E64" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F64" s="69" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G64" s="11">
         <v>2</v>
       </c>
       <c r="H64" s="12" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="B65" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C65" s="8" t="s">
         <v>260</v>
       </c>
-      <c r="B65" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="C65" s="8" t="s">
+      <c r="D65" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="D65" s="9" t="s">
-        <v>262</v>
-      </c>
       <c r="E65" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F65" s="69" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G65" s="11">
         <v>2</v>
       </c>
       <c r="H65" s="12" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C66" s="8" t="s">
         <v>264</v>
       </c>
-      <c r="B66" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="C66" s="8" t="s">
+      <c r="D66" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="D66" s="9" t="s">
+      <c r="E66" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F66" s="70" t="s">
         <v>266</v>
-      </c>
-      <c r="E66" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F66" s="70" t="s">
-        <v>267</v>
       </c>
       <c r="G66" s="11">
         <v>3</v>
       </c>
       <c r="H66" s="12" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C67" s="8" t="s">
         <v>269</v>
       </c>
-      <c r="B67" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="C67" s="8" t="s">
+      <c r="D67" s="9" t="s">
         <v>270</v>
       </c>
-      <c r="D67" s="9" t="s">
+      <c r="E67" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F67" s="11" t="s">
         <v>271</v>
-      </c>
-      <c r="E67" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F67" s="11" t="s">
-        <v>272</v>
       </c>
       <c r="G67" s="11">
         <v>5</v>
       </c>
       <c r="H67" s="12" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C68" s="8" t="s">
         <v>274</v>
       </c>
-      <c r="B68" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="C68" s="8" t="s">
+      <c r="D68" s="9" t="s">
         <v>275</v>
       </c>
-      <c r="D68" s="9" t="s">
-        <v>276</v>
-      </c>
       <c r="E68" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F68" s="69" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G68" s="11">
         <v>2</v>
       </c>
       <c r="H68" s="12" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="B69" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C69" s="71" t="s">
         <v>278</v>
       </c>
-      <c r="B69" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="C69" s="71" t="s">
+      <c r="D69" s="72" t="s">
         <v>279</v>
-      </c>
-      <c r="D69" s="72" t="s">
-        <v>280</v>
       </c>
       <c r="E69" s="55"/>
       <c r="F69" s="56" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="G69" s="56">
         <v>5</v>
       </c>
       <c r="H69" s="57" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C70" s="71" t="s">
         <v>282</v>
       </c>
-      <c r="B70" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="C70" s="71" t="s">
+      <c r="D70" s="72" t="s">
         <v>283</v>
-      </c>
-      <c r="D70" s="72" t="s">
-        <v>284</v>
       </c>
       <c r="E70" s="55"/>
       <c r="F70" s="73" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G70" s="56">
         <v>5</v>
       </c>
       <c r="H70" s="57" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="B71" s="74" t="s">
+        <v>246</v>
+      </c>
+      <c r="C71" s="75" t="s">
         <v>286</v>
       </c>
-      <c r="B71" s="74" t="s">
-        <v>247</v>
-      </c>
-      <c r="C71" s="75" t="s">
+      <c r="D71" s="76" t="s">
         <v>287</v>
-      </c>
-      <c r="D71" s="76" t="s">
-        <v>288</v>
       </c>
       <c r="E71" s="77"/>
       <c r="F71" s="69" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G71" s="78">
         <v>7</v>
       </c>
       <c r="H71" s="52" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="B72" s="60" t="s">
         <v>290</v>
       </c>
-      <c r="B72" s="60" t="s">
+      <c r="C72" s="60" t="s">
         <v>291</v>
       </c>
-      <c r="C72" s="60" t="s">
+      <c r="D72" s="28" t="s">
         <v>292</v>
       </c>
-      <c r="D72" s="28" t="s">
+      <c r="E72" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F72" s="79" t="s">
         <v>293</v>
-      </c>
-      <c r="E72" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F72" s="79" t="s">
-        <v>294</v>
       </c>
       <c r="G72" s="11">
         <v>20</v>
       </c>
       <c r="H72" s="12" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="B73" s="60" t="s">
+        <v>290</v>
+      </c>
+      <c r="C73" s="60" t="s">
         <v>296</v>
       </c>
-      <c r="B73" s="60" t="s">
-        <v>291</v>
-      </c>
-      <c r="C73" s="60" t="s">
+      <c r="D73" s="28" t="s">
         <v>297</v>
       </c>
-      <c r="D73" s="28" t="s">
-        <v>298</v>
-      </c>
       <c r="E73" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F73" s="79" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G73" s="11">
         <v>10</v>
       </c>
       <c r="H73" s="12" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="B74" s="60" t="s">
+        <v>290</v>
+      </c>
+      <c r="C74" s="18" t="s">
         <v>300</v>
       </c>
-      <c r="B74" s="60" t="s">
-        <v>291</v>
-      </c>
-      <c r="C74" s="18" t="s">
+      <c r="D74" s="28" t="s">
         <v>301</v>
       </c>
-      <c r="D74" s="28" t="s">
-        <v>302</v>
-      </c>
       <c r="E74" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F74" s="79" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G74" s="11">
         <v>6</v>
       </c>
       <c r="H74" s="12" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="B75" s="60" t="s">
+        <v>290</v>
+      </c>
+      <c r="C75" s="60" t="s">
         <v>304</v>
       </c>
-      <c r="B75" s="60" t="s">
-        <v>291</v>
-      </c>
-      <c r="C75" s="60" t="s">
+      <c r="D75" s="28" t="s">
         <v>305</v>
       </c>
-      <c r="D75" s="28" t="s">
+      <c r="E75" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F75" s="80" t="s">
         <v>306</v>
-      </c>
-      <c r="E75" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F75" s="80" t="s">
-        <v>307</v>
       </c>
       <c r="G75" s="11">
         <v>8</v>
       </c>
       <c r="H75" s="12" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="B76" s="60" t="s">
+        <v>290</v>
+      </c>
+      <c r="C76" s="59" t="s">
         <v>309</v>
       </c>
-      <c r="B76" s="60" t="s">
-        <v>291</v>
-      </c>
-      <c r="C76" s="59" t="s">
+      <c r="D76" s="19" t="s">
         <v>310</v>
       </c>
-      <c r="D76" s="19" t="s">
+      <c r="E76" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F76" s="81" t="s">
         <v>311</v>
-      </c>
-      <c r="E76" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F76" s="81" t="s">
-        <v>312</v>
       </c>
       <c r="G76" s="15">
         <v>6</v>
       </c>
       <c r="H76" s="16" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="B77" s="60" t="s">
+        <v>290</v>
+      </c>
+      <c r="C77" s="60" t="s">
         <v>314</v>
       </c>
-      <c r="B77" s="60" t="s">
-        <v>291</v>
-      </c>
-      <c r="C77" s="60" t="s">
+      <c r="D77" s="28" t="s">
         <v>315</v>
       </c>
-      <c r="D77" s="28" t="s">
-        <v>316</v>
-      </c>
       <c r="E77" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F77" s="79" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G77" s="11">
         <v>13</v>
       </c>
       <c r="H77" s="12" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="B78" s="60" t="s">
+        <v>290</v>
+      </c>
+      <c r="C78" s="60" t="s">
         <v>318</v>
       </c>
-      <c r="B78" s="60" t="s">
-        <v>291</v>
-      </c>
-      <c r="C78" s="60" t="s">
+      <c r="D78" s="28" t="s">
         <v>319</v>
       </c>
-      <c r="D78" s="28" t="s">
-        <v>320</v>
-      </c>
       <c r="E78" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F78" s="11" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G78" s="11">
         <v>12</v>
       </c>
       <c r="H78" s="12" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="B79" s="60" t="s">
+        <v>290</v>
+      </c>
+      <c r="C79" s="60" t="s">
         <v>322</v>
       </c>
-      <c r="B79" s="60" t="s">
-        <v>291</v>
-      </c>
-      <c r="C79" s="60" t="s">
+      <c r="D79" s="28" t="s">
         <v>323</v>
       </c>
-      <c r="D79" s="28" t="s">
-        <v>324</v>
-      </c>
       <c r="E79" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F79" s="79" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G79" s="11">
         <v>4</v>
       </c>
       <c r="H79" s="12" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="B80" s="60" t="s">
+        <v>290</v>
+      </c>
+      <c r="C80" s="60" t="s">
         <v>326</v>
       </c>
-      <c r="B80" s="60" t="s">
-        <v>291</v>
-      </c>
-      <c r="C80" s="60" t="s">
+      <c r="D80" s="28" t="s">
         <v>327</v>
       </c>
-      <c r="D80" s="28" t="s">
-        <v>328</v>
-      </c>
       <c r="E80" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F80" s="81" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="G80" s="11">
         <v>9</v>
       </c>
       <c r="H80" s="57" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
+        <v>329</v>
+      </c>
+      <c r="B81" s="8" t="s">
         <v>330</v>
       </c>
-      <c r="B81" s="8" t="s">
+      <c r="C81" s="8" t="s">
         <v>331</v>
       </c>
-      <c r="C81" s="8" t="s">
+      <c r="D81" s="9" t="s">
         <v>332</v>
-      </c>
-      <c r="D81" s="9" t="s">
-        <v>333</v>
       </c>
       <c r="E81" s="10" t="s">
         <v>0</v>
@@ -4775,429 +4775,429 @@
         <v>4</v>
       </c>
       <c r="H81" s="12" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="B82" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="C82" s="8" t="s">
         <v>335</v>
       </c>
-      <c r="B82" s="8" t="s">
-        <v>331</v>
-      </c>
-      <c r="C82" s="8" t="s">
+      <c r="D82" s="14" t="s">
         <v>336</v>
       </c>
-      <c r="D82" s="14" t="s">
-        <v>337</v>
-      </c>
       <c r="E82" s="2" t="s">
         <v>0</v>
       </c>
       <c r="F82" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G82" s="15">
         <v>3</v>
       </c>
       <c r="H82" s="16" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="B83" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="C83" s="8" t="s">
         <v>339</v>
       </c>
-      <c r="B83" s="8" t="s">
-        <v>331</v>
-      </c>
-      <c r="C83" s="8" t="s">
+      <c r="D83" s="14" t="s">
         <v>340</v>
       </c>
-      <c r="D83" s="14" t="s">
-        <v>341</v>
-      </c>
       <c r="E83" s="2" t="s">
         <v>0</v>
       </c>
       <c r="F83" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G83" s="15">
         <v>3</v>
       </c>
       <c r="H83" s="16" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" s="7" t="s">
+        <v>342</v>
+      </c>
+      <c r="B84" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="C84" s="8" t="s">
         <v>343</v>
       </c>
-      <c r="B84" s="8" t="s">
-        <v>331</v>
-      </c>
-      <c r="C84" s="8" t="s">
+      <c r="D84" s="9" t="s">
         <v>344</v>
       </c>
-      <c r="D84" s="9" t="s">
-        <v>345</v>
-      </c>
       <c r="E84" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F84" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G84" s="11">
         <v>3</v>
       </c>
       <c r="H84" s="12" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" s="7" t="s">
+        <v>346</v>
+      </c>
+      <c r="B85" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="C85" s="74" t="s">
         <v>347</v>
       </c>
-      <c r="B85" s="8" t="s">
-        <v>331</v>
-      </c>
-      <c r="C85" s="74" t="s">
+      <c r="D85" s="83" t="s">
         <v>348</v>
       </c>
-      <c r="D85" s="83" t="s">
-        <v>349</v>
-      </c>
       <c r="E85" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F85" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G85" s="11">
         <v>6</v>
       </c>
       <c r="H85" s="12" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="B86" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="C86" s="8" t="s">
         <v>351</v>
       </c>
-      <c r="B86" s="8" t="s">
-        <v>331</v>
-      </c>
-      <c r="C86" s="8" t="s">
+      <c r="D86" s="9" t="s">
         <v>352</v>
       </c>
-      <c r="D86" s="9" t="s">
-        <v>353</v>
-      </c>
       <c r="E86" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F86" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G86" s="11">
         <v>3</v>
       </c>
       <c r="H86" s="12" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="7" t="s">
+        <v>354</v>
+      </c>
+      <c r="B87" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="C87" s="8" t="s">
         <v>355</v>
       </c>
-      <c r="B87" s="8" t="s">
-        <v>331</v>
-      </c>
-      <c r="C87" s="8" t="s">
+      <c r="D87" s="9" t="s">
         <v>356</v>
       </c>
-      <c r="D87" s="9" t="s">
-        <v>357</v>
-      </c>
       <c r="E87" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F87" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G87" s="11">
         <v>6</v>
       </c>
       <c r="H87" s="12" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="C88" s="31" t="s">
         <v>359</v>
       </c>
-      <c r="B88" s="8" t="s">
-        <v>331</v>
-      </c>
-      <c r="C88" s="31" t="s">
+      <c r="D88" s="9" t="s">
         <v>360</v>
       </c>
-      <c r="D88" s="9" t="s">
-        <v>361</v>
-      </c>
       <c r="E88" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F88" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G88" s="11">
         <v>5</v>
       </c>
       <c r="H88" s="12" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="B89" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="C89" s="31" t="s">
         <v>363</v>
       </c>
-      <c r="B89" s="8" t="s">
-        <v>331</v>
-      </c>
-      <c r="C89" s="31" t="s">
+      <c r="D89" s="9" t="s">
         <v>364</v>
       </c>
-      <c r="D89" s="9" t="s">
-        <v>365</v>
-      </c>
       <c r="E89" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F89" s="11" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="G89" s="11">
         <v>4</v>
       </c>
       <c r="H89" s="57" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="I89" s="84"/>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="7" t="s">
+        <v>366</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="C90" s="31" t="s">
         <v>367</v>
       </c>
-      <c r="B90" s="8" t="s">
-        <v>331</v>
-      </c>
-      <c r="C90" s="31" t="s">
+      <c r="D90" s="9" t="s">
         <v>368</v>
-      </c>
-      <c r="D90" s="9" t="s">
-        <v>369</v>
       </c>
       <c r="E90" s="10"/>
       <c r="F90" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G90" s="11">
         <v>3</v>
       </c>
       <c r="H90" s="12" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="85" t="s">
+        <v>370</v>
+      </c>
+      <c r="B91" s="74" t="s">
+        <v>330</v>
+      </c>
+      <c r="C91" s="86" t="s">
         <v>371</v>
       </c>
-      <c r="B91" s="74" t="s">
-        <v>331</v>
-      </c>
-      <c r="C91" s="86" t="s">
+      <c r="D91" s="83" t="s">
         <v>372</v>
-      </c>
-      <c r="D91" s="83" t="s">
-        <v>373</v>
       </c>
       <c r="E91" s="77"/>
       <c r="F91" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G91" s="78">
         <v>4</v>
       </c>
       <c r="H91" s="52" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="I91" s="84"/>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="7" t="s">
+        <v>374</v>
+      </c>
+      <c r="B92" s="60" t="s">
         <v>375</v>
       </c>
-      <c r="B92" s="60" t="s">
+      <c r="C92" s="18" t="s">
         <v>376</v>
       </c>
-      <c r="C92" s="18" t="s">
+      <c r="D92" s="28" t="s">
         <v>377</v>
       </c>
-      <c r="D92" s="28" t="s">
+      <c r="E92" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F92" s="11" t="s">
         <v>378</v>
-      </c>
-      <c r="E92" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F92" s="11" t="s">
-        <v>379</v>
       </c>
       <c r="G92" s="11">
         <v>3</v>
       </c>
       <c r="H92" s="12" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="B93" s="60" t="s">
+        <v>375</v>
+      </c>
+      <c r="C93" s="60" t="s">
         <v>381</v>
       </c>
-      <c r="B93" s="60" t="s">
-        <v>376</v>
-      </c>
-      <c r="C93" s="60" t="s">
+      <c r="D93" s="28" t="s">
         <v>382</v>
       </c>
-      <c r="D93" s="28" t="s">
-        <v>383</v>
-      </c>
       <c r="E93" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F93" s="11" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="G93" s="11">
         <v>3</v>
       </c>
       <c r="H93" s="12" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="B94" s="60" t="s">
+        <v>375</v>
+      </c>
+      <c r="C94" s="60" t="s">
         <v>385</v>
       </c>
-      <c r="B94" s="60" t="s">
-        <v>376</v>
-      </c>
-      <c r="C94" s="60" t="s">
+      <c r="D94" s="28" t="s">
         <v>386</v>
       </c>
-      <c r="D94" s="28" t="s">
-        <v>387</v>
-      </c>
       <c r="E94" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F94" s="11" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="G94" s="11">
         <v>3</v>
       </c>
       <c r="H94" s="12" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="7" t="s">
+        <v>388</v>
+      </c>
+      <c r="B95" s="60" t="s">
+        <v>375</v>
+      </c>
+      <c r="C95" s="60" t="s">
         <v>389</v>
       </c>
-      <c r="B95" s="60" t="s">
-        <v>376</v>
-      </c>
-      <c r="C95" s="60" t="s">
+      <c r="D95" s="28" t="s">
         <v>390</v>
       </c>
-      <c r="D95" s="28" t="s">
-        <v>391</v>
-      </c>
       <c r="E95" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F95" s="11" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="G95" s="11">
         <v>3</v>
       </c>
       <c r="H95" s="12" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="B96" s="60" t="s">
+        <v>375</v>
+      </c>
+      <c r="C96" s="59" t="s">
         <v>393</v>
       </c>
-      <c r="B96" s="60" t="s">
-        <v>376</v>
-      </c>
-      <c r="C96" s="59" t="s">
+      <c r="D96" s="19" t="s">
         <v>394</v>
       </c>
-      <c r="D96" s="19" t="s">
-        <v>395</v>
-      </c>
       <c r="E96" s="2" t="s">
         <v>0</v>
       </c>
       <c r="F96" s="15" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="G96" s="15">
         <v>3</v>
       </c>
       <c r="H96" s="16" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" s="7" t="s">
+        <v>396</v>
+      </c>
+      <c r="B97" s="60" t="s">
+        <v>375</v>
+      </c>
+      <c r="C97" s="65" t="s">
         <v>397</v>
       </c>
-      <c r="B97" s="60" t="s">
-        <v>376</v>
-      </c>
-      <c r="C97" s="65" t="s">
+      <c r="D97" s="28" t="s">
         <v>398</v>
       </c>
-      <c r="D97" s="28" t="s">
-        <v>399</v>
-      </c>
       <c r="E97" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F97" s="11" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="G97" s="11">
         <v>3</v>
       </c>
       <c r="H97" s="12" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" s="7" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B98" s="60" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C98" s="60" t="s">
         <v>42</v>
@@ -5209,7 +5209,7 @@
         <v>0</v>
       </c>
       <c r="F98" s="11" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="G98" s="11">
         <v>3</v>
@@ -5220,810 +5220,810 @@
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" s="7" t="s">
+        <v>401</v>
+      </c>
+      <c r="B99" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="B99" s="8" t="s">
+      <c r="C99" s="8" t="s">
         <v>403</v>
       </c>
-      <c r="C99" s="8" t="s">
+      <c r="D99" s="9" t="s">
         <v>404</v>
       </c>
-      <c r="D99" s="9" t="s">
-        <v>405</v>
-      </c>
       <c r="E99" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F99" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G99" s="11">
         <v>4</v>
       </c>
       <c r="H99" s="12" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" s="7" t="s">
+        <v>406</v>
+      </c>
+      <c r="B100" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="C100" s="8" t="s">
         <v>407</v>
       </c>
-      <c r="B100" s="8" t="s">
-        <v>403</v>
-      </c>
-      <c r="C100" s="8" t="s">
+      <c r="D100" s="9" t="s">
         <v>408</v>
       </c>
-      <c r="D100" s="9" t="s">
-        <v>409</v>
-      </c>
       <c r="E100" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F100" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G100" s="11">
         <v>3</v>
       </c>
       <c r="H100" s="12" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" s="7" t="s">
+        <v>410</v>
+      </c>
+      <c r="B101" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="C101" s="8" t="s">
         <v>411</v>
       </c>
-      <c r="B101" s="8" t="s">
-        <v>403</v>
-      </c>
-      <c r="C101" s="8" t="s">
+      <c r="D101" s="9" t="s">
         <v>412</v>
       </c>
-      <c r="D101" s="9" t="s">
-        <v>413</v>
-      </c>
       <c r="E101" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F101" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G101" s="11">
         <v>2</v>
       </c>
       <c r="H101" s="12" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" s="7" t="s">
+        <v>414</v>
+      </c>
+      <c r="B102" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="C102" s="8" t="s">
         <v>415</v>
       </c>
-      <c r="B102" s="8" t="s">
-        <v>403</v>
-      </c>
-      <c r="C102" s="8" t="s">
+      <c r="D102" s="9" t="s">
         <v>416</v>
       </c>
-      <c r="D102" s="9" t="s">
-        <v>417</v>
-      </c>
       <c r="E102" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F102" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G102" s="11">
         <v>2</v>
       </c>
       <c r="H102" s="12" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" s="7" t="s">
+        <v>418</v>
+      </c>
+      <c r="B103" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="C103" s="8" t="s">
         <v>419</v>
       </c>
-      <c r="B103" s="8" t="s">
-        <v>403</v>
-      </c>
-      <c r="C103" s="8" t="s">
+      <c r="D103" s="9" t="s">
         <v>420</v>
       </c>
-      <c r="D103" s="9" t="s">
-        <v>421</v>
-      </c>
       <c r="E103" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F103" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G103" s="11">
         <v>2</v>
       </c>
       <c r="H103" s="12" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" s="7" t="s">
+        <v>422</v>
+      </c>
+      <c r="B104" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="C104" s="8" t="s">
         <v>423</v>
       </c>
-      <c r="B104" s="8" t="s">
-        <v>403</v>
-      </c>
-      <c r="C104" s="8" t="s">
+      <c r="D104" s="9" t="s">
         <v>424</v>
       </c>
-      <c r="D104" s="9" t="s">
-        <v>425</v>
-      </c>
       <c r="E104" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F104" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G104" s="11">
         <v>3</v>
       </c>
       <c r="H104" s="12" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" s="7" t="s">
+        <v>426</v>
+      </c>
+      <c r="B105" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="C105" s="8" t="s">
         <v>427</v>
       </c>
-      <c r="B105" s="8" t="s">
-        <v>403</v>
-      </c>
-      <c r="C105" s="8" t="s">
+      <c r="D105" s="9" t="s">
         <v>428</v>
       </c>
-      <c r="D105" s="9" t="s">
-        <v>429</v>
-      </c>
       <c r="E105" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F105" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G105" s="11">
         <v>3</v>
       </c>
       <c r="H105" s="12" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="B106" s="74" t="s">
+        <v>402</v>
+      </c>
+      <c r="C106" s="74" t="s">
         <v>431</v>
       </c>
-      <c r="B106" s="74" t="s">
-        <v>403</v>
-      </c>
-      <c r="C106" s="74" t="s">
+      <c r="D106" s="83" t="s">
         <v>432</v>
       </c>
-      <c r="D106" s="83" t="s">
-        <v>433</v>
-      </c>
       <c r="E106" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F106" s="70" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G106" s="11">
         <v>2</v>
       </c>
       <c r="H106" s="12" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="B107" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="C107" s="8" t="s">
         <v>435</v>
       </c>
-      <c r="B107" s="8" t="s">
-        <v>403</v>
-      </c>
-      <c r="C107" s="8" t="s">
+      <c r="D107" s="9" t="s">
         <v>436</v>
       </c>
-      <c r="D107" s="9" t="s">
-        <v>437</v>
-      </c>
       <c r="E107" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F107" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G107" s="11">
         <v>4</v>
       </c>
       <c r="H107" s="12" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" s="7" t="s">
+        <v>438</v>
+      </c>
+      <c r="B108" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="C108" s="8" t="s">
         <v>439</v>
       </c>
-      <c r="B108" s="8" t="s">
-        <v>403</v>
-      </c>
-      <c r="C108" s="8" t="s">
+      <c r="D108" s="9" t="s">
         <v>440</v>
       </c>
-      <c r="D108" s="9" t="s">
-        <v>441</v>
-      </c>
       <c r="E108" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F108" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G108" s="11">
         <v>3</v>
       </c>
       <c r="H108" s="12" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" s="7" t="s">
+        <v>442</v>
+      </c>
+      <c r="B109" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="C109" s="8" t="s">
         <v>443</v>
       </c>
-      <c r="B109" s="8" t="s">
-        <v>403</v>
-      </c>
-      <c r="C109" s="8" t="s">
+      <c r="D109" s="9" t="s">
         <v>444</v>
-      </c>
-      <c r="D109" s="9" t="s">
-        <v>445</v>
       </c>
       <c r="E109" s="10"/>
       <c r="F109" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G109" s="11">
         <v>4</v>
       </c>
       <c r="H109" s="12" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" s="7" t="s">
+        <v>446</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="C110" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="B110" s="8" t="s">
-        <v>403</v>
-      </c>
-      <c r="C110" s="8" t="s">
+      <c r="D110" s="9" t="s">
         <v>448</v>
-      </c>
-      <c r="D110" s="9" t="s">
-        <v>449</v>
       </c>
       <c r="E110" s="10"/>
       <c r="F110" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G110" s="11">
         <v>5</v>
       </c>
       <c r="H110" s="12" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" s="7" t="s">
+        <v>450</v>
+      </c>
+      <c r="B111" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="C111" s="31" t="s">
         <v>451</v>
       </c>
-      <c r="B111" s="8" t="s">
-        <v>403</v>
-      </c>
-      <c r="C111" s="31" t="s">
+      <c r="D111" s="9" t="s">
         <v>452</v>
-      </c>
-      <c r="D111" s="9" t="s">
-        <v>453</v>
       </c>
       <c r="E111" s="10"/>
       <c r="F111" s="80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G111" s="11">
         <v>4</v>
       </c>
       <c r="H111" s="12" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112" s="87" t="s">
+        <v>454</v>
+      </c>
+      <c r="B112" s="60" t="s">
         <v>455</v>
       </c>
-      <c r="B112" s="60" t="s">
+      <c r="C112" s="59" t="s">
         <v>456</v>
       </c>
-      <c r="C112" s="59" t="s">
+      <c r="D112" s="28" t="s">
         <v>457</v>
       </c>
-      <c r="D112" s="28" t="s">
+      <c r="E112" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F112" s="11" t="s">
         <v>458</v>
-      </c>
-      <c r="E112" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F112" s="11" t="s">
-        <v>459</v>
       </c>
       <c r="G112" s="11">
         <v>2</v>
       </c>
       <c r="H112" s="57" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113" s="87" t="s">
+        <v>460</v>
+      </c>
+      <c r="B113" s="60" t="s">
+        <v>455</v>
+      </c>
+      <c r="C113" s="60" t="s">
         <v>461</v>
       </c>
-      <c r="B113" s="60" t="s">
-        <v>456</v>
-      </c>
-      <c r="C113" s="60" t="s">
+      <c r="D113" s="19" t="s">
         <v>462</v>
       </c>
-      <c r="D113" s="19" t="s">
+      <c r="E113" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F113" s="15" t="s">
         <v>463</v>
-      </c>
-      <c r="E113" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F113" s="15" t="s">
-        <v>464</v>
       </c>
       <c r="G113" s="15">
         <v>2</v>
       </c>
       <c r="H113" s="16" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114" s="87" t="s">
+        <v>465</v>
+      </c>
+      <c r="B114" s="60" t="s">
+        <v>455</v>
+      </c>
+      <c r="C114" s="60" t="s">
         <v>466</v>
       </c>
-      <c r="B114" s="60" t="s">
-        <v>456</v>
-      </c>
-      <c r="C114" s="60" t="s">
+      <c r="D114" s="19" t="s">
         <v>467</v>
       </c>
-      <c r="D114" s="19" t="s">
-        <v>468</v>
-      </c>
       <c r="E114" s="2" t="s">
         <v>0</v>
       </c>
       <c r="F114" s="15" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="G114" s="15">
         <v>2</v>
       </c>
       <c r="H114" s="16" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115" s="87" t="s">
+        <v>469</v>
+      </c>
+      <c r="B115" s="60" t="s">
+        <v>455</v>
+      </c>
+      <c r="C115" s="60" t="s">
         <v>470</v>
       </c>
-      <c r="B115" s="60" t="s">
-        <v>456</v>
-      </c>
-      <c r="C115" s="60" t="s">
+      <c r="D115" s="19" t="s">
         <v>471</v>
       </c>
-      <c r="D115" s="19" t="s">
-        <v>472</v>
-      </c>
       <c r="E115" s="2" t="s">
         <v>0</v>
       </c>
       <c r="F115" s="15" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="G115" s="15">
         <v>2</v>
       </c>
       <c r="H115" s="16" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116" s="87" t="s">
+        <v>473</v>
+      </c>
+      <c r="B116" s="60" t="s">
+        <v>455</v>
+      </c>
+      <c r="C116" s="60" t="s">
         <v>474</v>
       </c>
-      <c r="B116" s="60" t="s">
-        <v>456</v>
-      </c>
-      <c r="C116" s="60" t="s">
+      <c r="D116" s="28" t="s">
         <v>475</v>
       </c>
-      <c r="D116" s="28" t="s">
-        <v>476</v>
-      </c>
       <c r="E116" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F116" s="11" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="G116" s="11">
         <v>2</v>
       </c>
       <c r="H116" s="12" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117" s="87" t="s">
+        <v>477</v>
+      </c>
+      <c r="B117" s="60" t="s">
+        <v>455</v>
+      </c>
+      <c r="C117" s="60" t="s">
         <v>478</v>
       </c>
-      <c r="B117" s="60" t="s">
-        <v>456</v>
-      </c>
-      <c r="C117" s="60" t="s">
+      <c r="D117" s="28" t="s">
         <v>479</v>
       </c>
-      <c r="D117" s="28" t="s">
-        <v>480</v>
-      </c>
       <c r="E117" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F117" s="11" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="G117" s="11">
         <v>2</v>
       </c>
       <c r="H117" s="12" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118" s="87" t="s">
+        <v>481</v>
+      </c>
+      <c r="B118" s="60" t="s">
+        <v>455</v>
+      </c>
+      <c r="C118" s="60" t="s">
         <v>482</v>
       </c>
-      <c r="B118" s="60" t="s">
-        <v>456</v>
-      </c>
-      <c r="C118" s="60" t="s">
+      <c r="D118" s="28" t="s">
         <v>483</v>
       </c>
-      <c r="D118" s="28" t="s">
-        <v>484</v>
-      </c>
       <c r="E118" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F118" s="11" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="G118" s="11">
         <v>2</v>
       </c>
       <c r="H118" s="12" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A119" s="87" t="s">
+        <v>485</v>
+      </c>
+      <c r="B119" s="60" t="s">
+        <v>455</v>
+      </c>
+      <c r="C119" s="60" t="s">
         <v>486</v>
       </c>
-      <c r="B119" s="60" t="s">
-        <v>456</v>
-      </c>
-      <c r="C119" s="60" t="s">
+      <c r="D119" s="28" t="s">
         <v>487</v>
       </c>
-      <c r="D119" s="28" t="s">
-        <v>488</v>
-      </c>
       <c r="E119" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F119" s="11" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="G119" s="11">
         <v>3</v>
       </c>
       <c r="H119" s="12" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120" s="87" t="s">
+        <v>489</v>
+      </c>
+      <c r="B120" s="60" t="s">
+        <v>455</v>
+      </c>
+      <c r="C120" s="60" t="s">
         <v>490</v>
       </c>
-      <c r="B120" s="60" t="s">
-        <v>456</v>
-      </c>
-      <c r="C120" s="60" t="s">
+      <c r="D120" s="28" t="s">
         <v>491</v>
       </c>
-      <c r="D120" s="28" t="s">
-        <v>492</v>
-      </c>
       <c r="E120" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F120" s="11" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="G120" s="11">
         <v>2</v>
       </c>
       <c r="H120" s="12" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A121" s="87" t="s">
+        <v>493</v>
+      </c>
+      <c r="B121" s="60" t="s">
+        <v>455</v>
+      </c>
+      <c r="C121" s="60" t="s">
         <v>494</v>
       </c>
-      <c r="B121" s="60" t="s">
-        <v>456</v>
-      </c>
-      <c r="C121" s="60" t="s">
+      <c r="D121" s="28" t="s">
         <v>495</v>
       </c>
-      <c r="D121" s="28" t="s">
-        <v>496</v>
-      </c>
       <c r="E121" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F121" s="11" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="G121" s="11">
         <v>1</v>
       </c>
       <c r="H121" s="12" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122" s="87" t="s">
+        <v>497</v>
+      </c>
+      <c r="B122" s="60" t="s">
+        <v>455</v>
+      </c>
+      <c r="C122" s="60" t="s">
         <v>498</v>
       </c>
-      <c r="B122" s="60" t="s">
-        <v>456</v>
-      </c>
-      <c r="C122" s="60" t="s">
+      <c r="D122" s="28" t="s">
         <v>499</v>
       </c>
-      <c r="D122" s="28" t="s">
+      <c r="E122" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F122" s="11" t="s">
         <v>500</v>
-      </c>
-      <c r="E122" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F122" s="11" t="s">
-        <v>501</v>
       </c>
       <c r="G122" s="11">
         <v>2</v>
       </c>
       <c r="H122" s="12" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="123" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A123" s="87" t="s">
+        <v>502</v>
+      </c>
+      <c r="B123" s="60" t="s">
+        <v>455</v>
+      </c>
+      <c r="C123" s="60" t="s">
         <v>503</v>
       </c>
-      <c r="B123" s="60" t="s">
-        <v>456</v>
-      </c>
-      <c r="C123" s="60" t="s">
+      <c r="D123" s="28" t="s">
         <v>504</v>
       </c>
-      <c r="D123" s="28" t="s">
-        <v>505</v>
-      </c>
       <c r="E123" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F123" s="11" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="G123" s="11">
         <v>2</v>
       </c>
       <c r="H123" s="12" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="124" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A124" s="87" t="s">
+        <v>506</v>
+      </c>
+      <c r="B124" s="60" t="s">
+        <v>455</v>
+      </c>
+      <c r="C124" s="60" t="s">
         <v>507</v>
       </c>
-      <c r="B124" s="60" t="s">
-        <v>456</v>
-      </c>
-      <c r="C124" s="60" t="s">
+      <c r="D124" s="28" t="s">
         <v>508</v>
       </c>
-      <c r="D124" s="28" t="s">
-        <v>509</v>
-      </c>
       <c r="E124" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F124" s="11" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="G124" s="11">
         <v>2</v>
       </c>
       <c r="H124" s="12" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A125" s="87" t="s">
+        <v>510</v>
+      </c>
+      <c r="B125" s="60" t="s">
+        <v>455</v>
+      </c>
+      <c r="C125" s="60" t="s">
         <v>511</v>
       </c>
-      <c r="B125" s="60" t="s">
-        <v>456</v>
-      </c>
-      <c r="C125" s="60" t="s">
+      <c r="D125" s="28" t="s">
         <v>512</v>
       </c>
-      <c r="D125" s="28" t="s">
-        <v>513</v>
-      </c>
       <c r="E125" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F125" s="11" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="G125" s="11">
         <v>1</v>
       </c>
       <c r="H125" s="12" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A126" s="87" t="s">
+        <v>514</v>
+      </c>
+      <c r="B126" s="60" t="s">
+        <v>455</v>
+      </c>
+      <c r="C126" s="60" t="s">
         <v>515</v>
       </c>
-      <c r="B126" s="60" t="s">
-        <v>456</v>
-      </c>
-      <c r="C126" s="60" t="s">
-        <v>516</v>
-      </c>
       <c r="D126" s="28" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="E126" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F126" s="11" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="G126" s="11">
         <v>2</v>
       </c>
       <c r="H126" s="12" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A127" s="87" t="s">
+        <v>517</v>
+      </c>
+      <c r="B127" s="60" t="s">
+        <v>455</v>
+      </c>
+      <c r="C127" s="60" t="s">
         <v>518</v>
       </c>
-      <c r="B127" s="60" t="s">
-        <v>456</v>
-      </c>
-      <c r="C127" s="60" t="s">
+      <c r="D127" s="28" t="s">
         <v>519</v>
       </c>
-      <c r="D127" s="28" t="s">
-        <v>520</v>
-      </c>
       <c r="E127" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F127" s="11" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="G127" s="11">
         <v>3</v>
       </c>
       <c r="H127" s="12" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
     <row r="128" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A128" s="87" t="s">
+        <v>521</v>
+      </c>
+      <c r="B128" s="60" t="s">
+        <v>455</v>
+      </c>
+      <c r="C128" s="18" t="s">
         <v>522</v>
       </c>
-      <c r="B128" s="60" t="s">
-        <v>456</v>
-      </c>
-      <c r="C128" s="18" t="s">
+      <c r="D128" s="28" t="s">
         <v>523</v>
       </c>
-      <c r="D128" s="28" t="s">
-        <v>524</v>
-      </c>
       <c r="E128" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F128" s="11" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="G128" s="11">
         <v>4</v>
       </c>
       <c r="H128" s="12" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A129" s="87" t="s">
+        <v>525</v>
+      </c>
+      <c r="B129" s="60" t="s">
+        <v>455</v>
+      </c>
+      <c r="C129" s="59" t="s">
         <v>526</v>
       </c>
-      <c r="B129" s="60" t="s">
-        <v>456</v>
-      </c>
-      <c r="C129" s="59" t="s">
+      <c r="D129" s="19" t="s">
         <v>527</v>
       </c>
-      <c r="D129" s="19" t="s">
-        <v>528</v>
-      </c>
       <c r="E129" s="2" t="s">
         <v>0</v>
       </c>
       <c r="F129" s="15" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="G129" s="15">
         <v>3</v>
       </c>
       <c r="H129" s="16" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
     </row>
     <row r="130" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A130" s="87" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B130" s="60" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="C130" s="18" t="s">
         <v>42</v>
@@ -6046,42 +6046,42 @@
     </row>
     <row r="131" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A131" s="7" t="s">
+        <v>530</v>
+      </c>
+      <c r="B131" s="8" t="s">
         <v>531</v>
       </c>
-      <c r="B131" s="8" t="s">
+      <c r="C131" s="88" t="s">
         <v>532</v>
       </c>
-      <c r="C131" s="88" t="s">
+      <c r="D131" s="14" t="s">
         <v>533</v>
       </c>
-      <c r="D131" s="14" t="s">
+      <c r="E131" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F131" s="15" t="s">
         <v>534</v>
-      </c>
-      <c r="E131" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F131" s="15" t="s">
-        <v>535</v>
       </c>
       <c r="G131" s="15">
         <v>3</v>
       </c>
       <c r="H131" s="16" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
     </row>
     <row r="132" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A132" s="7" t="s">
+        <v>536</v>
+      </c>
+      <c r="B132" s="8" t="s">
+        <v>531</v>
+      </c>
+      <c r="C132" s="9" t="s">
         <v>537</v>
       </c>
-      <c r="B132" s="8" t="s">
-        <v>532</v>
-      </c>
-      <c r="C132" s="9" t="s">
+      <c r="D132" s="9" t="s">
         <v>538</v>
-      </c>
-      <c r="D132" s="9" t="s">
-        <v>539</v>
       </c>
       <c r="E132" s="10" t="s">
         <v>11</v>
@@ -6099,16 +6099,16 @@
     </row>
     <row r="133" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A133" s="7" t="s">
+        <v>539</v>
+      </c>
+      <c r="B133" s="8" t="s">
+        <v>531</v>
+      </c>
+      <c r="C133" s="9" t="s">
         <v>540</v>
       </c>
-      <c r="B133" s="8" t="s">
-        <v>532</v>
-      </c>
-      <c r="C133" s="9" t="s">
+      <c r="D133" s="9" t="s">
         <v>541</v>
-      </c>
-      <c r="D133" s="9" t="s">
-        <v>542</v>
       </c>
       <c r="E133" s="10" t="s">
         <v>11</v>
@@ -6123,88 +6123,88 @@
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A134" s="7" t="s">
+        <v>542</v>
+      </c>
+      <c r="B134" s="8" t="s">
+        <v>531</v>
+      </c>
+      <c r="C134" s="8" t="s">
         <v>543</v>
       </c>
-      <c r="B134" s="8" t="s">
-        <v>532</v>
-      </c>
-      <c r="C134" s="8" t="s">
+      <c r="D134" s="9" t="s">
         <v>544</v>
       </c>
-      <c r="D134" s="9" t="s">
+      <c r="E134" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F134" s="11" t="s">
         <v>545</v>
-      </c>
-      <c r="E134" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F134" s="11" t="s">
-        <v>546</v>
       </c>
       <c r="G134" s="11"/>
       <c r="H134" s="12" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A135" s="7" t="s">
+        <v>547</v>
+      </c>
+      <c r="B135" s="8" t="s">
+        <v>531</v>
+      </c>
+      <c r="C135" s="8" t="s">
         <v>548</v>
       </c>
-      <c r="B135" s="8" t="s">
-        <v>532</v>
-      </c>
-      <c r="C135" s="8" t="s">
+      <c r="D135" s="9" t="s">
         <v>549</v>
       </c>
-      <c r="D135" s="9" t="s">
-        <v>550</v>
-      </c>
       <c r="E135" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F135" s="11" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="G135" s="11"/>
       <c r="H135" s="12" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="136" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A136" s="7" t="s">
+        <v>551</v>
+      </c>
+      <c r="B136" s="8" t="s">
+        <v>531</v>
+      </c>
+      <c r="C136" s="8" t="s">
         <v>552</v>
       </c>
-      <c r="B136" s="8" t="s">
-        <v>532</v>
-      </c>
-      <c r="C136" s="8" t="s">
+      <c r="D136" s="9" t="s">
         <v>553</v>
       </c>
-      <c r="D136" s="9" t="s">
+      <c r="E136" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F136" s="11" t="s">
         <v>554</v>
-      </c>
-      <c r="E136" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F136" s="11" t="s">
-        <v>555</v>
       </c>
       <c r="G136" s="11"/>
       <c r="H136" s="12" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
     </row>
     <row r="137" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A137" s="7" t="s">
+        <v>556</v>
+      </c>
+      <c r="B137" s="8" t="s">
+        <v>531</v>
+      </c>
+      <c r="C137" s="9" t="s">
         <v>557</v>
       </c>
-      <c r="B137" s="8" t="s">
-        <v>532</v>
-      </c>
-      <c r="C137" s="9" t="s">
+      <c r="D137" s="9" t="s">
         <v>558</v>
-      </c>
-      <c r="D137" s="9" t="s">
-        <v>559</v>
       </c>
       <c r="E137" s="10" t="s">
         <v>11</v>
@@ -6219,16 +6219,16 @@
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A138" s="7" t="s">
+        <v>559</v>
+      </c>
+      <c r="B138" s="8" t="s">
+        <v>531</v>
+      </c>
+      <c r="C138" s="48" t="s">
         <v>560</v>
       </c>
-      <c r="B138" s="8" t="s">
-        <v>532</v>
-      </c>
-      <c r="C138" s="48" t="s">
+      <c r="D138" s="9" t="s">
         <v>561</v>
-      </c>
-      <c r="D138" s="9" t="s">
-        <v>562</v>
       </c>
       <c r="E138" s="10" t="s">
         <v>11</v>
@@ -6243,26 +6243,26 @@
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A139" s="7" t="s">
+        <v>562</v>
+      </c>
+      <c r="B139" s="8" t="s">
+        <v>531</v>
+      </c>
+      <c r="C139" s="88" t="s">
         <v>563</v>
       </c>
-      <c r="B139" s="8" t="s">
-        <v>532</v>
-      </c>
-      <c r="C139" s="88" t="s">
+      <c r="D139" s="14" t="s">
         <v>564</v>
       </c>
-      <c r="D139" s="14" t="s">
+      <c r="E139" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F139" s="15" t="s">
         <v>565</v>
-      </c>
-      <c r="E139" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F139" s="15" t="s">
-        <v>566</v>
       </c>
       <c r="G139" s="15"/>
       <c r="H139" s="16" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="140" spans="1:8" x14ac:dyDescent="0.25">
@@ -6287,17 +6287,17 @@
     </row>
     <row r="143" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B143" s="6" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="144" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B144" s="6" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="145" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B145" s="6" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
after adding feature to import 145s from FAA list.
</commit_message>
<xml_diff>
--- a/assets/db_code lookups/Business Category and Search.xlsx
+++ b/assets/db_code lookups/Business Category and Search.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jared\source\repos\data_sync_desktop\assets\db_code lookups\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{363760AF-45C9-4EAA-B5ED-174C56455814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D0646650-61EA-421D-B218-E0AC24CF4999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F6BDE4B6-EF96-429D-83BC-A8CA702EE26E}"/>
+    <workbookView xWindow="4575" yWindow="840" windowWidth="21600" windowHeight="13140" xr2:uid="{F6BDE4B6-EF96-429D-83BC-A8CA702EE26E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$139</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -417,9 +418,6 @@
   </si>
   <si>
     <t>P147</t>
-  </si>
-  <si>
-    <t>maintenance training | maintenance school | AP school | A&amp;P school|aircraft maintenance training| airframe and pwerplant school| A and P school</t>
   </si>
   <si>
     <t>05F</t>
@@ -1781,6 +1779,9 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>maintenance training | maintenance school | AP school | A&amp;P school|aircraft maintenance training| airframe and powerplant school| A and P school</t>
   </si>
 </sst>
 </file>
@@ -3143,7 +3144,7 @@
         <v>75</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>0</v>
@@ -3493,21 +3494,21 @@
         <v>8</v>
       </c>
       <c r="H31" s="12" t="s">
-        <v>126</v>
+        <v>569</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B32" s="30" t="s">
         <v>106</v>
       </c>
       <c r="C32" s="31" t="s">
+        <v>127</v>
+      </c>
+      <c r="D32" s="9" t="s">
         <v>128</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>129</v>
       </c>
       <c r="E32" s="10" t="s">
         <v>0</v>
@@ -3519,64 +3520,64 @@
         <v>3</v>
       </c>
       <c r="H32" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B33" s="30" t="s">
         <v>106</v>
       </c>
       <c r="C33" s="48" t="s">
+        <v>131</v>
+      </c>
+      <c r="D33" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="D33" s="9" t="s">
+      <c r="E33" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F33" s="49" t="s">
         <v>133</v>
-      </c>
-      <c r="E33" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F33" s="49" t="s">
-        <v>134</v>
       </c>
       <c r="G33" s="11">
         <v>4</v>
       </c>
       <c r="H33" s="12" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B34" s="30" t="s">
         <v>106</v>
       </c>
       <c r="C34" s="31" t="s">
+        <v>136</v>
+      </c>
+      <c r="D34" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="D34" s="9" t="s">
-        <v>138</v>
-      </c>
       <c r="E34" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F34" s="49" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G34" s="11">
         <v>3</v>
       </c>
       <c r="H34" s="12" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B35" s="30" t="s">
         <v>106</v>
@@ -3602,16 +3603,16 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B36" s="30" t="s">
         <v>106</v>
       </c>
       <c r="C36" s="50" t="s">
+        <v>141</v>
+      </c>
+      <c r="D36" s="51" t="s">
         <v>142</v>
-      </c>
-      <c r="D36" s="51" t="s">
-        <v>143</v>
       </c>
       <c r="E36" s="10"/>
       <c r="F36" s="47" t="s">
@@ -3621,21 +3622,21 @@
         <v>3</v>
       </c>
       <c r="H36" s="12" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B37" s="30" t="s">
         <v>106</v>
       </c>
       <c r="C37" s="50" t="s">
+        <v>145</v>
+      </c>
+      <c r="D37" s="51" t="s">
         <v>146</v>
-      </c>
-      <c r="D37" s="51" t="s">
-        <v>147</v>
       </c>
       <c r="E37" s="10"/>
       <c r="F37" s="47" t="s">
@@ -3645,21 +3646,21 @@
         <v>4</v>
       </c>
       <c r="H37" s="52" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B38" s="30" t="s">
         <v>106</v>
       </c>
       <c r="C38" s="50" t="s">
+        <v>149</v>
+      </c>
+      <c r="D38" s="51" t="s">
         <v>150</v>
-      </c>
-      <c r="D38" s="51" t="s">
-        <v>151</v>
       </c>
       <c r="E38" s="10"/>
       <c r="F38" s="47" t="s">
@@ -3669,21 +3670,21 @@
         <v>6</v>
       </c>
       <c r="H38" s="12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B39" s="30" t="s">
         <v>106</v>
       </c>
       <c r="C39" s="53" t="s">
+        <v>153</v>
+      </c>
+      <c r="D39" s="54" t="s">
         <v>154</v>
-      </c>
-      <c r="D39" s="54" t="s">
-        <v>155</v>
       </c>
       <c r="E39" s="55"/>
       <c r="F39" s="47" t="s">
@@ -3693,538 +3694,538 @@
         <v>11</v>
       </c>
       <c r="H39" s="57" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="B40" s="17" t="s">
         <v>157</v>
       </c>
-      <c r="B40" s="17" t="s">
+      <c r="C40" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="C40" s="18" t="s">
+      <c r="D40" s="28" t="s">
         <v>159</v>
       </c>
-      <c r="D40" s="28" t="s">
+      <c r="E40" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F40" s="58" t="s">
         <v>160</v>
-      </c>
-      <c r="E40" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F40" s="58" t="s">
-        <v>161</v>
       </c>
       <c r="G40" s="11">
         <v>9</v>
       </c>
       <c r="H40" s="12" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="B41" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="C41" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="B41" s="17" t="s">
-        <v>158</v>
-      </c>
-      <c r="C41" s="18" t="s">
+      <c r="D41" s="28" t="s">
         <v>164</v>
       </c>
-      <c r="D41" s="28" t="s">
-        <v>165</v>
-      </c>
       <c r="E41" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F41" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G41" s="11">
         <v>12</v>
       </c>
       <c r="H41" s="12" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="B42" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="C42" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="B42" s="17" t="s">
-        <v>158</v>
-      </c>
-      <c r="C42" s="18" t="s">
+      <c r="D42" s="28" t="s">
         <v>168</v>
       </c>
-      <c r="D42" s="28" t="s">
-        <v>169</v>
-      </c>
       <c r="E42" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F42" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G42" s="11">
         <v>7</v>
       </c>
       <c r="H42" s="12" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="B43" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="C43" s="29" t="s">
         <v>171</v>
       </c>
-      <c r="B43" s="17" t="s">
-        <v>158</v>
-      </c>
-      <c r="C43" s="29" t="s">
+      <c r="D43" s="28" t="s">
         <v>172</v>
       </c>
-      <c r="D43" s="28" t="s">
-        <v>173</v>
-      </c>
       <c r="E43" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F43" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G43" s="11">
         <v>7</v>
       </c>
       <c r="H43" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="B44" s="59" t="s">
+        <v>157</v>
+      </c>
+      <c r="C44" s="60" t="s">
         <v>175</v>
       </c>
-      <c r="B44" s="59" t="s">
-        <v>158</v>
-      </c>
-      <c r="C44" s="60" t="s">
+      <c r="D44" s="19" t="s">
         <v>176</v>
       </c>
-      <c r="D44" s="19" t="s">
-        <v>177</v>
-      </c>
       <c r="E44" s="2" t="s">
         <v>0</v>
       </c>
       <c r="F44" s="61" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G44" s="15">
         <v>5</v>
       </c>
       <c r="H44" s="16" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="B45" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C45" s="60" t="s">
         <v>179</v>
       </c>
-      <c r="B45" s="60" t="s">
-        <v>158</v>
-      </c>
-      <c r="C45" s="60" t="s">
+      <c r="D45" s="28" t="s">
         <v>180</v>
       </c>
-      <c r="D45" s="28" t="s">
-        <v>181</v>
-      </c>
       <c r="E45" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F45" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G45" s="11">
         <v>5</v>
       </c>
       <c r="H45" s="12" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="B46" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C46" s="60" t="s">
         <v>183</v>
       </c>
-      <c r="B46" s="60" t="s">
-        <v>158</v>
-      </c>
-      <c r="C46" s="60" t="s">
+      <c r="D46" s="28" t="s">
         <v>184</v>
       </c>
-      <c r="D46" s="28" t="s">
-        <v>185</v>
-      </c>
       <c r="E46" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F46" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G46" s="11">
         <v>2</v>
       </c>
       <c r="H46" s="12" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="B47" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C47" s="60" t="s">
         <v>187</v>
       </c>
-      <c r="B47" s="60" t="s">
-        <v>158</v>
-      </c>
-      <c r="C47" s="60" t="s">
+      <c r="D47" s="28" t="s">
         <v>188</v>
       </c>
-      <c r="D47" s="28" t="s">
-        <v>189</v>
-      </c>
       <c r="E47" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F47" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G47" s="11">
         <v>13</v>
       </c>
       <c r="H47" s="12" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="B48" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C48" s="60" t="s">
         <v>191</v>
       </c>
-      <c r="B48" s="60" t="s">
-        <v>158</v>
-      </c>
-      <c r="C48" s="60" t="s">
+      <c r="D48" s="28" t="s">
         <v>192</v>
       </c>
-      <c r="D48" s="28" t="s">
-        <v>193</v>
-      </c>
       <c r="E48" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F48" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G48" s="11">
         <v>4</v>
       </c>
       <c r="H48" s="12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="B49" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C49" s="60" t="s">
         <v>195</v>
       </c>
-      <c r="B49" s="60" t="s">
-        <v>158</v>
-      </c>
-      <c r="C49" s="60" t="s">
+      <c r="D49" s="28" t="s">
         <v>196</v>
       </c>
-      <c r="D49" s="28" t="s">
-        <v>197</v>
-      </c>
       <c r="E49" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F49" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G49" s="11">
         <v>2</v>
       </c>
       <c r="H49" s="12" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="B50" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C50" s="60" t="s">
         <v>199</v>
       </c>
-      <c r="B50" s="60" t="s">
-        <v>158</v>
-      </c>
-      <c r="C50" s="60" t="s">
+      <c r="D50" s="28" t="s">
         <v>200</v>
       </c>
-      <c r="D50" s="28" t="s">
-        <v>201</v>
-      </c>
       <c r="E50" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F50" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G50" s="11">
         <v>2</v>
       </c>
       <c r="H50" s="12" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="B51" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C51" s="60" t="s">
         <v>203</v>
       </c>
-      <c r="B51" s="60" t="s">
-        <v>158</v>
-      </c>
-      <c r="C51" s="60" t="s">
+      <c r="D51" s="28" t="s">
         <v>204</v>
       </c>
-      <c r="D51" s="28" t="s">
-        <v>205</v>
-      </c>
       <c r="E51" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F51" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G51" s="11">
         <v>4</v>
       </c>
       <c r="H51" s="12" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="B52" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C52" s="60" t="s">
         <v>207</v>
       </c>
-      <c r="B52" s="60" t="s">
-        <v>158</v>
-      </c>
-      <c r="C52" s="60" t="s">
+      <c r="D52" s="28" t="s">
         <v>208</v>
       </c>
-      <c r="D52" s="28" t="s">
-        <v>209</v>
-      </c>
       <c r="E52" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F52" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G52" s="11">
         <v>4</v>
       </c>
       <c r="H52" s="12" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="B53" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C53" s="60" t="s">
         <v>211</v>
       </c>
-      <c r="B53" s="60" t="s">
-        <v>158</v>
-      </c>
-      <c r="C53" s="60" t="s">
+      <c r="D53" s="28" t="s">
         <v>212</v>
       </c>
-      <c r="D53" s="28" t="s">
-        <v>213</v>
-      </c>
       <c r="E53" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F53" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G53" s="11">
         <v>3</v>
       </c>
       <c r="H53" s="12" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="B54" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C54" s="60" t="s">
         <v>215</v>
       </c>
-      <c r="B54" s="60" t="s">
-        <v>158</v>
-      </c>
-      <c r="C54" s="60" t="s">
+      <c r="D54" s="28" t="s">
         <v>216</v>
       </c>
-      <c r="D54" s="28" t="s">
-        <v>217</v>
-      </c>
       <c r="E54" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F54" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G54" s="11">
         <v>6</v>
       </c>
       <c r="H54" s="12" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="B55" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C55" s="60" t="s">
         <v>219</v>
       </c>
-      <c r="B55" s="60" t="s">
-        <v>158</v>
-      </c>
-      <c r="C55" s="60" t="s">
+      <c r="D55" s="28" t="s">
         <v>220</v>
       </c>
-      <c r="D55" s="28" t="s">
-        <v>221</v>
-      </c>
       <c r="E55" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F55" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G55" s="11">
         <v>4</v>
       </c>
       <c r="H55" s="12" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="B56" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C56" s="60" t="s">
         <v>223</v>
       </c>
-      <c r="B56" s="60" t="s">
-        <v>158</v>
-      </c>
-      <c r="C56" s="60" t="s">
+      <c r="D56" s="28" t="s">
         <v>224</v>
       </c>
-      <c r="D56" s="28" t="s">
-        <v>225</v>
-      </c>
       <c r="E56" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F56" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G56" s="11">
         <v>3</v>
       </c>
       <c r="H56" s="52" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="B57" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C57" s="60" t="s">
         <v>227</v>
       </c>
-      <c r="B57" s="60" t="s">
-        <v>158</v>
-      </c>
-      <c r="C57" s="60" t="s">
+      <c r="D57" s="28" t="s">
         <v>228</v>
       </c>
-      <c r="D57" s="28" t="s">
-        <v>229</v>
-      </c>
       <c r="E57" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F57" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G57" s="11">
         <v>3</v>
       </c>
       <c r="H57" s="12" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="B58" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C58" s="60" t="s">
         <v>231</v>
       </c>
-      <c r="B58" s="60" t="s">
-        <v>158</v>
-      </c>
-      <c r="C58" s="60" t="s">
+      <c r="D58" s="28" t="s">
         <v>232</v>
       </c>
-      <c r="D58" s="28" t="s">
-        <v>233</v>
-      </c>
       <c r="E58" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F58" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G58" s="11">
         <v>3</v>
       </c>
       <c r="H58" s="12" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="B59" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C59" s="60" t="s">
         <v>235</v>
       </c>
-      <c r="B59" s="60" t="s">
-        <v>158</v>
-      </c>
-      <c r="C59" s="60" t="s">
+      <c r="D59" s="28" t="s">
         <v>236</v>
       </c>
-      <c r="D59" s="28" t="s">
-        <v>237</v>
-      </c>
       <c r="E59" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F59" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G59" s="11">
         <v>2</v>
       </c>
       <c r="H59" s="57" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="B60" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C60" s="62" t="s">
         <v>239</v>
-      </c>
-      <c r="B60" s="60" t="s">
-        <v>158</v>
-      </c>
-      <c r="C60" s="62" t="s">
-        <v>240</v>
       </c>
       <c r="D60" s="63" t="s">
         <v>43</v>
@@ -4242,528 +4243,528 @@
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="B61" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C61" s="65" t="s">
         <v>241</v>
       </c>
-      <c r="B61" s="60" t="s">
-        <v>158</v>
-      </c>
-      <c r="C61" s="65" t="s">
+      <c r="D61" s="66" t="s">
         <v>242</v>
-      </c>
-      <c r="D61" s="66" t="s">
-        <v>243</v>
       </c>
       <c r="E61" s="67"/>
       <c r="F61" s="68" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G61" s="64">
         <v>4</v>
       </c>
       <c r="H61" s="52" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="B62" s="8" t="s">
         <v>245</v>
       </c>
-      <c r="B62" s="8" t="s">
+      <c r="C62" s="8" t="s">
         <v>246</v>
       </c>
-      <c r="C62" s="8" t="s">
+      <c r="D62" s="9" t="s">
         <v>247</v>
       </c>
-      <c r="D62" s="9" t="s">
+      <c r="E62" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F62" s="69" t="s">
         <v>248</v>
-      </c>
-      <c r="E62" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F62" s="69" t="s">
-        <v>249</v>
       </c>
       <c r="G62" s="11">
         <v>7</v>
       </c>
       <c r="H62" s="12" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="B63" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="C63" s="8" t="s">
         <v>251</v>
       </c>
-      <c r="B63" s="8" t="s">
-        <v>246</v>
-      </c>
-      <c r="C63" s="8" t="s">
+      <c r="D63" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="D63" s="9" t="s">
-        <v>253</v>
-      </c>
       <c r="E63" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F63" s="69" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G63" s="11">
         <v>4</v>
       </c>
       <c r="H63" s="12" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="C64" s="8" t="s">
         <v>255</v>
       </c>
-      <c r="B64" s="8" t="s">
-        <v>246</v>
-      </c>
-      <c r="C64" s="8" t="s">
+      <c r="D64" s="9" t="s">
         <v>256</v>
       </c>
-      <c r="D64" s="9" t="s">
-        <v>257</v>
-      </c>
       <c r="E64" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F64" s="69" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G64" s="11">
         <v>2</v>
       </c>
       <c r="H64" s="12" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="B65" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="C65" s="8" t="s">
         <v>259</v>
       </c>
-      <c r="B65" s="8" t="s">
-        <v>246</v>
-      </c>
-      <c r="C65" s="8" t="s">
+      <c r="D65" s="9" t="s">
         <v>260</v>
       </c>
-      <c r="D65" s="9" t="s">
-        <v>261</v>
-      </c>
       <c r="E65" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F65" s="69" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G65" s="11">
         <v>2</v>
       </c>
       <c r="H65" s="12" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="C66" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="B66" s="8" t="s">
-        <v>246</v>
-      </c>
-      <c r="C66" s="8" t="s">
+      <c r="D66" s="9" t="s">
         <v>264</v>
       </c>
-      <c r="D66" s="9" t="s">
+      <c r="E66" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F66" s="70" t="s">
         <v>265</v>
-      </c>
-      <c r="E66" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F66" s="70" t="s">
-        <v>266</v>
       </c>
       <c r="G66" s="11">
         <v>3</v>
       </c>
       <c r="H66" s="12" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="C67" s="8" t="s">
         <v>268</v>
       </c>
-      <c r="B67" s="8" t="s">
-        <v>246</v>
-      </c>
-      <c r="C67" s="8" t="s">
+      <c r="D67" s="9" t="s">
         <v>269</v>
       </c>
-      <c r="D67" s="9" t="s">
+      <c r="E67" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F67" s="11" t="s">
         <v>270</v>
-      </c>
-      <c r="E67" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F67" s="11" t="s">
-        <v>271</v>
       </c>
       <c r="G67" s="11">
         <v>5</v>
       </c>
       <c r="H67" s="12" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="C68" s="8" t="s">
         <v>273</v>
       </c>
-      <c r="B68" s="8" t="s">
-        <v>246</v>
-      </c>
-      <c r="C68" s="8" t="s">
+      <c r="D68" s="9" t="s">
         <v>274</v>
       </c>
-      <c r="D68" s="9" t="s">
-        <v>275</v>
-      </c>
       <c r="E68" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F68" s="69" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G68" s="11">
         <v>2</v>
       </c>
       <c r="H68" s="12" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="B69" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="C69" s="71" t="s">
         <v>277</v>
       </c>
-      <c r="B69" s="8" t="s">
-        <v>246</v>
-      </c>
-      <c r="C69" s="71" t="s">
+      <c r="D69" s="72" t="s">
         <v>278</v>
-      </c>
-      <c r="D69" s="72" t="s">
-        <v>279</v>
       </c>
       <c r="E69" s="55"/>
       <c r="F69" s="56" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="G69" s="56">
         <v>5</v>
       </c>
       <c r="H69" s="57" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="C70" s="71" t="s">
         <v>281</v>
       </c>
-      <c r="B70" s="8" t="s">
-        <v>246</v>
-      </c>
-      <c r="C70" s="71" t="s">
+      <c r="D70" s="72" t="s">
         <v>282</v>
-      </c>
-      <c r="D70" s="72" t="s">
-        <v>283</v>
       </c>
       <c r="E70" s="55"/>
       <c r="F70" s="73" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G70" s="56">
         <v>5</v>
       </c>
       <c r="H70" s="57" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="B71" s="74" t="s">
+        <v>245</v>
+      </c>
+      <c r="C71" s="75" t="s">
         <v>285</v>
       </c>
-      <c r="B71" s="74" t="s">
-        <v>246</v>
-      </c>
-      <c r="C71" s="75" t="s">
+      <c r="D71" s="76" t="s">
         <v>286</v>
-      </c>
-      <c r="D71" s="76" t="s">
-        <v>287</v>
       </c>
       <c r="E71" s="77"/>
       <c r="F71" s="69" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G71" s="78">
         <v>7</v>
       </c>
       <c r="H71" s="52" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="B72" s="60" t="s">
         <v>289</v>
       </c>
-      <c r="B72" s="60" t="s">
+      <c r="C72" s="60" t="s">
         <v>290</v>
       </c>
-      <c r="C72" s="60" t="s">
+      <c r="D72" s="28" t="s">
         <v>291</v>
       </c>
-      <c r="D72" s="28" t="s">
+      <c r="E72" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F72" s="79" t="s">
         <v>292</v>
-      </c>
-      <c r="E72" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F72" s="79" t="s">
-        <v>293</v>
       </c>
       <c r="G72" s="11">
         <v>20</v>
       </c>
       <c r="H72" s="12" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="B73" s="60" t="s">
+        <v>289</v>
+      </c>
+      <c r="C73" s="60" t="s">
         <v>295</v>
       </c>
-      <c r="B73" s="60" t="s">
-        <v>290</v>
-      </c>
-      <c r="C73" s="60" t="s">
+      <c r="D73" s="28" t="s">
         <v>296</v>
       </c>
-      <c r="D73" s="28" t="s">
-        <v>297</v>
-      </c>
       <c r="E73" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F73" s="79" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G73" s="11">
         <v>10</v>
       </c>
       <c r="H73" s="12" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="B74" s="60" t="s">
+        <v>289</v>
+      </c>
+      <c r="C74" s="18" t="s">
         <v>299</v>
       </c>
-      <c r="B74" s="60" t="s">
-        <v>290</v>
-      </c>
-      <c r="C74" s="18" t="s">
+      <c r="D74" s="28" t="s">
         <v>300</v>
       </c>
-      <c r="D74" s="28" t="s">
-        <v>301</v>
-      </c>
       <c r="E74" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F74" s="79" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G74" s="11">
         <v>6</v>
       </c>
       <c r="H74" s="12" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="B75" s="60" t="s">
+        <v>289</v>
+      </c>
+      <c r="C75" s="60" t="s">
         <v>303</v>
       </c>
-      <c r="B75" s="60" t="s">
-        <v>290</v>
-      </c>
-      <c r="C75" s="60" t="s">
+      <c r="D75" s="28" t="s">
         <v>304</v>
       </c>
-      <c r="D75" s="28" t="s">
+      <c r="E75" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F75" s="80" t="s">
         <v>305</v>
-      </c>
-      <c r="E75" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F75" s="80" t="s">
-        <v>306</v>
       </c>
       <c r="G75" s="11">
         <v>8</v>
       </c>
       <c r="H75" s="12" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" s="7" t="s">
+        <v>307</v>
+      </c>
+      <c r="B76" s="60" t="s">
+        <v>289</v>
+      </c>
+      <c r="C76" s="59" t="s">
         <v>308</v>
       </c>
-      <c r="B76" s="60" t="s">
-        <v>290</v>
-      </c>
-      <c r="C76" s="59" t="s">
+      <c r="D76" s="19" t="s">
         <v>309</v>
       </c>
-      <c r="D76" s="19" t="s">
+      <c r="E76" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F76" s="81" t="s">
         <v>310</v>
-      </c>
-      <c r="E76" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F76" s="81" t="s">
-        <v>311</v>
       </c>
       <c r="G76" s="15">
         <v>6</v>
       </c>
       <c r="H76" s="16" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="B77" s="60" t="s">
+        <v>289</v>
+      </c>
+      <c r="C77" s="60" t="s">
         <v>313</v>
       </c>
-      <c r="B77" s="60" t="s">
-        <v>290</v>
-      </c>
-      <c r="C77" s="60" t="s">
+      <c r="D77" s="28" t="s">
         <v>314</v>
       </c>
-      <c r="D77" s="28" t="s">
-        <v>315</v>
-      </c>
       <c r="E77" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F77" s="79" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G77" s="11">
         <v>13</v>
       </c>
       <c r="H77" s="12" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="B78" s="60" t="s">
+        <v>289</v>
+      </c>
+      <c r="C78" s="60" t="s">
         <v>317</v>
       </c>
-      <c r="B78" s="60" t="s">
-        <v>290</v>
-      </c>
-      <c r="C78" s="60" t="s">
+      <c r="D78" s="28" t="s">
         <v>318</v>
       </c>
-      <c r="D78" s="28" t="s">
-        <v>319</v>
-      </c>
       <c r="E78" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F78" s="11" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G78" s="11">
         <v>12</v>
       </c>
       <c r="H78" s="12" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="B79" s="60" t="s">
+        <v>289</v>
+      </c>
+      <c r="C79" s="60" t="s">
         <v>321</v>
       </c>
-      <c r="B79" s="60" t="s">
-        <v>290</v>
-      </c>
-      <c r="C79" s="60" t="s">
+      <c r="D79" s="28" t="s">
         <v>322</v>
       </c>
-      <c r="D79" s="28" t="s">
-        <v>323</v>
-      </c>
       <c r="E79" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F79" s="79" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G79" s="11">
         <v>4</v>
       </c>
       <c r="H79" s="12" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="B80" s="60" t="s">
+        <v>289</v>
+      </c>
+      <c r="C80" s="60" t="s">
         <v>325</v>
       </c>
-      <c r="B80" s="60" t="s">
-        <v>290</v>
-      </c>
-      <c r="C80" s="60" t="s">
+      <c r="D80" s="28" t="s">
         <v>326</v>
       </c>
-      <c r="D80" s="28" t="s">
-        <v>327</v>
-      </c>
       <c r="E80" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F80" s="81" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="G80" s="11">
         <v>9</v>
       </c>
       <c r="H80" s="57" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="B81" s="8" t="s">
         <v>329</v>
       </c>
-      <c r="B81" s="8" t="s">
+      <c r="C81" s="8" t="s">
         <v>330</v>
       </c>
-      <c r="C81" s="8" t="s">
+      <c r="D81" s="9" t="s">
         <v>331</v>
-      </c>
-      <c r="D81" s="9" t="s">
-        <v>332</v>
       </c>
       <c r="E81" s="10" t="s">
         <v>0</v>
@@ -4775,429 +4776,429 @@
         <v>4</v>
       </c>
       <c r="H81" s="12" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="B82" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="C82" s="8" t="s">
         <v>334</v>
       </c>
-      <c r="B82" s="8" t="s">
-        <v>330</v>
-      </c>
-      <c r="C82" s="8" t="s">
+      <c r="D82" s="14" t="s">
         <v>335</v>
       </c>
-      <c r="D82" s="14" t="s">
-        <v>336</v>
-      </c>
       <c r="E82" s="2" t="s">
         <v>0</v>
       </c>
       <c r="F82" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G82" s="15">
         <v>3</v>
       </c>
       <c r="H82" s="16" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="B83" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="C83" s="8" t="s">
         <v>338</v>
       </c>
-      <c r="B83" s="8" t="s">
-        <v>330</v>
-      </c>
-      <c r="C83" s="8" t="s">
+      <c r="D83" s="14" t="s">
         <v>339</v>
       </c>
-      <c r="D83" s="14" t="s">
-        <v>340</v>
-      </c>
       <c r="E83" s="2" t="s">
         <v>0</v>
       </c>
       <c r="F83" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G83" s="15">
         <v>3</v>
       </c>
       <c r="H83" s="16" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" s="7" t="s">
+        <v>341</v>
+      </c>
+      <c r="B84" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="C84" s="8" t="s">
         <v>342</v>
       </c>
-      <c r="B84" s="8" t="s">
-        <v>330</v>
-      </c>
-      <c r="C84" s="8" t="s">
+      <c r="D84" s="9" t="s">
         <v>343</v>
       </c>
-      <c r="D84" s="9" t="s">
-        <v>344</v>
-      </c>
       <c r="E84" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F84" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G84" s="11">
         <v>3</v>
       </c>
       <c r="H84" s="12" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="B85" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="C85" s="74" t="s">
         <v>346</v>
       </c>
-      <c r="B85" s="8" t="s">
-        <v>330</v>
-      </c>
-      <c r="C85" s="74" t="s">
+      <c r="D85" s="83" t="s">
         <v>347</v>
       </c>
-      <c r="D85" s="83" t="s">
-        <v>348</v>
-      </c>
       <c r="E85" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F85" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G85" s="11">
         <v>6</v>
       </c>
       <c r="H85" s="12" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="7" t="s">
+        <v>349</v>
+      </c>
+      <c r="B86" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="C86" s="8" t="s">
         <v>350</v>
       </c>
-      <c r="B86" s="8" t="s">
-        <v>330</v>
-      </c>
-      <c r="C86" s="8" t="s">
+      <c r="D86" s="9" t="s">
         <v>351</v>
       </c>
-      <c r="D86" s="9" t="s">
-        <v>352</v>
-      </c>
       <c r="E86" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F86" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G86" s="11">
         <v>3</v>
       </c>
       <c r="H86" s="12" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="7" t="s">
+        <v>353</v>
+      </c>
+      <c r="B87" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="C87" s="8" t="s">
         <v>354</v>
       </c>
-      <c r="B87" s="8" t="s">
-        <v>330</v>
-      </c>
-      <c r="C87" s="8" t="s">
+      <c r="D87" s="9" t="s">
         <v>355</v>
       </c>
-      <c r="D87" s="9" t="s">
-        <v>356</v>
-      </c>
       <c r="E87" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F87" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G87" s="11">
         <v>6</v>
       </c>
       <c r="H87" s="12" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="7" t="s">
+        <v>357</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="C88" s="31" t="s">
         <v>358</v>
       </c>
-      <c r="B88" s="8" t="s">
-        <v>330</v>
-      </c>
-      <c r="C88" s="31" t="s">
+      <c r="D88" s="9" t="s">
         <v>359</v>
       </c>
-      <c r="D88" s="9" t="s">
-        <v>360</v>
-      </c>
       <c r="E88" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F88" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G88" s="11">
         <v>5</v>
       </c>
       <c r="H88" s="12" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="7" t="s">
+        <v>361</v>
+      </c>
+      <c r="B89" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="C89" s="31" t="s">
         <v>362</v>
       </c>
-      <c r="B89" s="8" t="s">
-        <v>330</v>
-      </c>
-      <c r="C89" s="31" t="s">
+      <c r="D89" s="9" t="s">
         <v>363</v>
       </c>
-      <c r="D89" s="9" t="s">
-        <v>364</v>
-      </c>
       <c r="E89" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F89" s="11" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="G89" s="11">
         <v>4</v>
       </c>
       <c r="H89" s="57" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="I89" s="84"/>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="7" t="s">
+        <v>365</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="C90" s="31" t="s">
         <v>366</v>
       </c>
-      <c r="B90" s="8" t="s">
-        <v>330</v>
-      </c>
-      <c r="C90" s="31" t="s">
+      <c r="D90" s="9" t="s">
         <v>367</v>
-      </c>
-      <c r="D90" s="9" t="s">
-        <v>368</v>
       </c>
       <c r="E90" s="10"/>
       <c r="F90" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G90" s="11">
         <v>3</v>
       </c>
       <c r="H90" s="12" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="85" t="s">
+        <v>369</v>
+      </c>
+      <c r="B91" s="74" t="s">
+        <v>329</v>
+      </c>
+      <c r="C91" s="86" t="s">
         <v>370</v>
       </c>
-      <c r="B91" s="74" t="s">
-        <v>330</v>
-      </c>
-      <c r="C91" s="86" t="s">
+      <c r="D91" s="83" t="s">
         <v>371</v>
-      </c>
-      <c r="D91" s="83" t="s">
-        <v>372</v>
       </c>
       <c r="E91" s="77"/>
       <c r="F91" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G91" s="78">
         <v>4</v>
       </c>
       <c r="H91" s="52" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="I91" s="84"/>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="B92" s="60" t="s">
         <v>374</v>
       </c>
-      <c r="B92" s="60" t="s">
+      <c r="C92" s="18" t="s">
         <v>375</v>
       </c>
-      <c r="C92" s="18" t="s">
+      <c r="D92" s="28" t="s">
         <v>376</v>
       </c>
-      <c r="D92" s="28" t="s">
+      <c r="E92" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F92" s="11" t="s">
         <v>377</v>
-      </c>
-      <c r="E92" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F92" s="11" t="s">
-        <v>378</v>
       </c>
       <c r="G92" s="11">
         <v>3</v>
       </c>
       <c r="H92" s="12" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="7" t="s">
+        <v>379</v>
+      </c>
+      <c r="B93" s="60" t="s">
+        <v>374</v>
+      </c>
+      <c r="C93" s="60" t="s">
         <v>380</v>
       </c>
-      <c r="B93" s="60" t="s">
-        <v>375</v>
-      </c>
-      <c r="C93" s="60" t="s">
+      <c r="D93" s="28" t="s">
         <v>381</v>
       </c>
-      <c r="D93" s="28" t="s">
-        <v>382</v>
-      </c>
       <c r="E93" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F93" s="11" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="G93" s="11">
         <v>3</v>
       </c>
       <c r="H93" s="12" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="B94" s="60" t="s">
+        <v>374</v>
+      </c>
+      <c r="C94" s="60" t="s">
         <v>384</v>
       </c>
-      <c r="B94" s="60" t="s">
-        <v>375</v>
-      </c>
-      <c r="C94" s="60" t="s">
+      <c r="D94" s="28" t="s">
         <v>385</v>
       </c>
-      <c r="D94" s="28" t="s">
-        <v>386</v>
-      </c>
       <c r="E94" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F94" s="11" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="G94" s="11">
         <v>3</v>
       </c>
       <c r="H94" s="12" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="B95" s="60" t="s">
+        <v>374</v>
+      </c>
+      <c r="C95" s="60" t="s">
         <v>388</v>
       </c>
-      <c r="B95" s="60" t="s">
-        <v>375</v>
-      </c>
-      <c r="C95" s="60" t="s">
+      <c r="D95" s="28" t="s">
         <v>389</v>
       </c>
-      <c r="D95" s="28" t="s">
-        <v>390</v>
-      </c>
       <c r="E95" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F95" s="11" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="G95" s="11">
         <v>3</v>
       </c>
       <c r="H95" s="12" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" s="7" t="s">
+        <v>391</v>
+      </c>
+      <c r="B96" s="60" t="s">
+        <v>374</v>
+      </c>
+      <c r="C96" s="59" t="s">
         <v>392</v>
       </c>
-      <c r="B96" s="60" t="s">
-        <v>375</v>
-      </c>
-      <c r="C96" s="59" t="s">
+      <c r="D96" s="19" t="s">
         <v>393</v>
       </c>
-      <c r="D96" s="19" t="s">
-        <v>394</v>
-      </c>
       <c r="E96" s="2" t="s">
         <v>0</v>
       </c>
       <c r="F96" s="15" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="G96" s="15">
         <v>3</v>
       </c>
       <c r="H96" s="16" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" s="7" t="s">
+        <v>395</v>
+      </c>
+      <c r="B97" s="60" t="s">
+        <v>374</v>
+      </c>
+      <c r="C97" s="65" t="s">
         <v>396</v>
       </c>
-      <c r="B97" s="60" t="s">
-        <v>375</v>
-      </c>
-      <c r="C97" s="65" t="s">
+      <c r="D97" s="28" t="s">
         <v>397</v>
       </c>
-      <c r="D97" s="28" t="s">
-        <v>398</v>
-      </c>
       <c r="E97" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F97" s="11" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="G97" s="11">
         <v>3</v>
       </c>
       <c r="H97" s="12" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" s="7" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B98" s="60" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C98" s="60" t="s">
         <v>42</v>
@@ -5209,7 +5210,7 @@
         <v>0</v>
       </c>
       <c r="F98" s="11" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="G98" s="11">
         <v>3</v>
@@ -5220,810 +5221,810 @@
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" s="7" t="s">
+        <v>400</v>
+      </c>
+      <c r="B99" s="8" t="s">
         <v>401</v>
       </c>
-      <c r="B99" s="8" t="s">
+      <c r="C99" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="C99" s="8" t="s">
+      <c r="D99" s="9" t="s">
         <v>403</v>
       </c>
-      <c r="D99" s="9" t="s">
-        <v>404</v>
-      </c>
       <c r="E99" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F99" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G99" s="11">
         <v>4</v>
       </c>
       <c r="H99" s="12" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" s="7" t="s">
+        <v>405</v>
+      </c>
+      <c r="B100" s="8" t="s">
+        <v>401</v>
+      </c>
+      <c r="C100" s="8" t="s">
         <v>406</v>
       </c>
-      <c r="B100" s="8" t="s">
-        <v>402</v>
-      </c>
-      <c r="C100" s="8" t="s">
+      <c r="D100" s="9" t="s">
         <v>407</v>
       </c>
-      <c r="D100" s="9" t="s">
-        <v>408</v>
-      </c>
       <c r="E100" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F100" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G100" s="11">
         <v>3</v>
       </c>
       <c r="H100" s="12" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="B101" s="8" t="s">
+        <v>401</v>
+      </c>
+      <c r="C101" s="8" t="s">
         <v>410</v>
       </c>
-      <c r="B101" s="8" t="s">
-        <v>402</v>
-      </c>
-      <c r="C101" s="8" t="s">
+      <c r="D101" s="9" t="s">
         <v>411</v>
       </c>
-      <c r="D101" s="9" t="s">
-        <v>412</v>
-      </c>
       <c r="E101" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F101" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G101" s="11">
         <v>2</v>
       </c>
       <c r="H101" s="12" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="B102" s="8" t="s">
+        <v>401</v>
+      </c>
+      <c r="C102" s="8" t="s">
         <v>414</v>
       </c>
-      <c r="B102" s="8" t="s">
-        <v>402</v>
-      </c>
-      <c r="C102" s="8" t="s">
+      <c r="D102" s="9" t="s">
         <v>415</v>
       </c>
-      <c r="D102" s="9" t="s">
-        <v>416</v>
-      </c>
       <c r="E102" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F102" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G102" s="11">
         <v>2</v>
       </c>
       <c r="H102" s="12" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" s="7" t="s">
+        <v>417</v>
+      </c>
+      <c r="B103" s="8" t="s">
+        <v>401</v>
+      </c>
+      <c r="C103" s="8" t="s">
         <v>418</v>
       </c>
-      <c r="B103" s="8" t="s">
-        <v>402</v>
-      </c>
-      <c r="C103" s="8" t="s">
+      <c r="D103" s="9" t="s">
         <v>419</v>
       </c>
-      <c r="D103" s="9" t="s">
-        <v>420</v>
-      </c>
       <c r="E103" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F103" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G103" s="11">
         <v>2</v>
       </c>
       <c r="H103" s="12" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" s="7" t="s">
+        <v>421</v>
+      </c>
+      <c r="B104" s="8" t="s">
+        <v>401</v>
+      </c>
+      <c r="C104" s="8" t="s">
         <v>422</v>
       </c>
-      <c r="B104" s="8" t="s">
-        <v>402</v>
-      </c>
-      <c r="C104" s="8" t="s">
+      <c r="D104" s="9" t="s">
         <v>423</v>
       </c>
-      <c r="D104" s="9" t="s">
-        <v>424</v>
-      </c>
       <c r="E104" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F104" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G104" s="11">
         <v>3</v>
       </c>
       <c r="H104" s="12" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" s="7" t="s">
+        <v>425</v>
+      </c>
+      <c r="B105" s="8" t="s">
+        <v>401</v>
+      </c>
+      <c r="C105" s="8" t="s">
         <v>426</v>
       </c>
-      <c r="B105" s="8" t="s">
-        <v>402</v>
-      </c>
-      <c r="C105" s="8" t="s">
+      <c r="D105" s="9" t="s">
         <v>427</v>
       </c>
-      <c r="D105" s="9" t="s">
-        <v>428</v>
-      </c>
       <c r="E105" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F105" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G105" s="11">
         <v>3</v>
       </c>
       <c r="H105" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" s="7" t="s">
+        <v>429</v>
+      </c>
+      <c r="B106" s="74" t="s">
+        <v>401</v>
+      </c>
+      <c r="C106" s="74" t="s">
         <v>430</v>
       </c>
-      <c r="B106" s="74" t="s">
-        <v>402</v>
-      </c>
-      <c r="C106" s="74" t="s">
+      <c r="D106" s="83" t="s">
         <v>431</v>
       </c>
-      <c r="D106" s="83" t="s">
-        <v>432</v>
-      </c>
       <c r="E106" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F106" s="70" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G106" s="11">
         <v>2</v>
       </c>
       <c r="H106" s="12" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" s="7" t="s">
+        <v>433</v>
+      </c>
+      <c r="B107" s="8" t="s">
+        <v>401</v>
+      </c>
+      <c r="C107" s="8" t="s">
         <v>434</v>
       </c>
-      <c r="B107" s="8" t="s">
-        <v>402</v>
-      </c>
-      <c r="C107" s="8" t="s">
+      <c r="D107" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="D107" s="9" t="s">
-        <v>436</v>
-      </c>
       <c r="E107" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F107" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G107" s="11">
         <v>4</v>
       </c>
       <c r="H107" s="12" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" s="7" t="s">
+        <v>437</v>
+      </c>
+      <c r="B108" s="8" t="s">
+        <v>401</v>
+      </c>
+      <c r="C108" s="8" t="s">
         <v>438</v>
       </c>
-      <c r="B108" s="8" t="s">
-        <v>402</v>
-      </c>
-      <c r="C108" s="8" t="s">
+      <c r="D108" s="9" t="s">
         <v>439</v>
       </c>
-      <c r="D108" s="9" t="s">
-        <v>440</v>
-      </c>
       <c r="E108" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F108" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G108" s="11">
         <v>3</v>
       </c>
       <c r="H108" s="12" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" s="7" t="s">
+        <v>441</v>
+      </c>
+      <c r="B109" s="8" t="s">
+        <v>401</v>
+      </c>
+      <c r="C109" s="8" t="s">
         <v>442</v>
       </c>
-      <c r="B109" s="8" t="s">
-        <v>402</v>
-      </c>
-      <c r="C109" s="8" t="s">
+      <c r="D109" s="9" t="s">
         <v>443</v>
-      </c>
-      <c r="D109" s="9" t="s">
-        <v>444</v>
       </c>
       <c r="E109" s="10"/>
       <c r="F109" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G109" s="11">
         <v>4</v>
       </c>
       <c r="H109" s="12" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" s="7" t="s">
+        <v>445</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>401</v>
+      </c>
+      <c r="C110" s="8" t="s">
         <v>446</v>
       </c>
-      <c r="B110" s="8" t="s">
-        <v>402</v>
-      </c>
-      <c r="C110" s="8" t="s">
+      <c r="D110" s="9" t="s">
         <v>447</v>
-      </c>
-      <c r="D110" s="9" t="s">
-        <v>448</v>
       </c>
       <c r="E110" s="10"/>
       <c r="F110" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G110" s="11">
         <v>5</v>
       </c>
       <c r="H110" s="12" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" s="7" t="s">
+        <v>449</v>
+      </c>
+      <c r="B111" s="8" t="s">
+        <v>401</v>
+      </c>
+      <c r="C111" s="31" t="s">
         <v>450</v>
       </c>
-      <c r="B111" s="8" t="s">
-        <v>402</v>
-      </c>
-      <c r="C111" s="31" t="s">
+      <c r="D111" s="9" t="s">
         <v>451</v>
-      </c>
-      <c r="D111" s="9" t="s">
-        <v>452</v>
       </c>
       <c r="E111" s="10"/>
       <c r="F111" s="80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G111" s="11">
         <v>4</v>
       </c>
       <c r="H111" s="12" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112" s="87" t="s">
+        <v>453</v>
+      </c>
+      <c r="B112" s="60" t="s">
         <v>454</v>
       </c>
-      <c r="B112" s="60" t="s">
+      <c r="C112" s="59" t="s">
         <v>455</v>
       </c>
-      <c r="C112" s="59" t="s">
+      <c r="D112" s="28" t="s">
         <v>456</v>
       </c>
-      <c r="D112" s="28" t="s">
+      <c r="E112" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F112" s="11" t="s">
         <v>457</v>
-      </c>
-      <c r="E112" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F112" s="11" t="s">
-        <v>458</v>
       </c>
       <c r="G112" s="11">
         <v>2</v>
       </c>
       <c r="H112" s="57" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113" s="87" t="s">
+        <v>459</v>
+      </c>
+      <c r="B113" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="C113" s="60" t="s">
         <v>460</v>
       </c>
-      <c r="B113" s="60" t="s">
-        <v>455</v>
-      </c>
-      <c r="C113" s="60" t="s">
+      <c r="D113" s="19" t="s">
         <v>461</v>
       </c>
-      <c r="D113" s="19" t="s">
+      <c r="E113" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F113" s="15" t="s">
         <v>462</v>
-      </c>
-      <c r="E113" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F113" s="15" t="s">
-        <v>463</v>
       </c>
       <c r="G113" s="15">
         <v>2</v>
       </c>
       <c r="H113" s="16" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114" s="87" t="s">
+        <v>464</v>
+      </c>
+      <c r="B114" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="C114" s="60" t="s">
         <v>465</v>
       </c>
-      <c r="B114" s="60" t="s">
-        <v>455</v>
-      </c>
-      <c r="C114" s="60" t="s">
+      <c r="D114" s="19" t="s">
         <v>466</v>
       </c>
-      <c r="D114" s="19" t="s">
-        <v>467</v>
-      </c>
       <c r="E114" s="2" t="s">
         <v>0</v>
       </c>
       <c r="F114" s="15" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="G114" s="15">
         <v>2</v>
       </c>
       <c r="H114" s="16" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115" s="87" t="s">
+        <v>468</v>
+      </c>
+      <c r="B115" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="C115" s="60" t="s">
         <v>469</v>
       </c>
-      <c r="B115" s="60" t="s">
-        <v>455</v>
-      </c>
-      <c r="C115" s="60" t="s">
+      <c r="D115" s="19" t="s">
         <v>470</v>
       </c>
-      <c r="D115" s="19" t="s">
-        <v>471</v>
-      </c>
       <c r="E115" s="2" t="s">
         <v>0</v>
       </c>
       <c r="F115" s="15" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="G115" s="15">
         <v>2</v>
       </c>
       <c r="H115" s="16" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116" s="87" t="s">
+        <v>472</v>
+      </c>
+      <c r="B116" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="C116" s="60" t="s">
         <v>473</v>
       </c>
-      <c r="B116" s="60" t="s">
-        <v>455</v>
-      </c>
-      <c r="C116" s="60" t="s">
+      <c r="D116" s="28" t="s">
         <v>474</v>
       </c>
-      <c r="D116" s="28" t="s">
-        <v>475</v>
-      </c>
       <c r="E116" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F116" s="11" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="G116" s="11">
         <v>2</v>
       </c>
       <c r="H116" s="12" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117" s="87" t="s">
+        <v>476</v>
+      </c>
+      <c r="B117" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="C117" s="60" t="s">
         <v>477</v>
       </c>
-      <c r="B117" s="60" t="s">
-        <v>455</v>
-      </c>
-      <c r="C117" s="60" t="s">
+      <c r="D117" s="28" t="s">
         <v>478</v>
       </c>
-      <c r="D117" s="28" t="s">
-        <v>479</v>
-      </c>
       <c r="E117" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F117" s="11" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="G117" s="11">
         <v>2</v>
       </c>
       <c r="H117" s="12" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118" s="87" t="s">
+        <v>480</v>
+      </c>
+      <c r="B118" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="C118" s="60" t="s">
         <v>481</v>
       </c>
-      <c r="B118" s="60" t="s">
-        <v>455</v>
-      </c>
-      <c r="C118" s="60" t="s">
+      <c r="D118" s="28" t="s">
         <v>482</v>
       </c>
-      <c r="D118" s="28" t="s">
-        <v>483</v>
-      </c>
       <c r="E118" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F118" s="11" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="G118" s="11">
         <v>2</v>
       </c>
       <c r="H118" s="12" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A119" s="87" t="s">
+        <v>484</v>
+      </c>
+      <c r="B119" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="C119" s="60" t="s">
         <v>485</v>
       </c>
-      <c r="B119" s="60" t="s">
-        <v>455</v>
-      </c>
-      <c r="C119" s="60" t="s">
+      <c r="D119" s="28" t="s">
         <v>486</v>
       </c>
-      <c r="D119" s="28" t="s">
-        <v>487</v>
-      </c>
       <c r="E119" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F119" s="11" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="G119" s="11">
         <v>3</v>
       </c>
       <c r="H119" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120" s="87" t="s">
+        <v>488</v>
+      </c>
+      <c r="B120" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="C120" s="60" t="s">
         <v>489</v>
       </c>
-      <c r="B120" s="60" t="s">
-        <v>455</v>
-      </c>
-      <c r="C120" s="60" t="s">
+      <c r="D120" s="28" t="s">
         <v>490</v>
       </c>
-      <c r="D120" s="28" t="s">
-        <v>491</v>
-      </c>
       <c r="E120" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F120" s="11" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="G120" s="11">
         <v>2</v>
       </c>
       <c r="H120" s="12" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A121" s="87" t="s">
+        <v>492</v>
+      </c>
+      <c r="B121" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="C121" s="60" t="s">
         <v>493</v>
       </c>
-      <c r="B121" s="60" t="s">
-        <v>455</v>
-      </c>
-      <c r="C121" s="60" t="s">
+      <c r="D121" s="28" t="s">
         <v>494</v>
       </c>
-      <c r="D121" s="28" t="s">
-        <v>495</v>
-      </c>
       <c r="E121" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F121" s="11" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="G121" s="11">
         <v>1</v>
       </c>
       <c r="H121" s="12" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122" s="87" t="s">
+        <v>496</v>
+      </c>
+      <c r="B122" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="C122" s="60" t="s">
         <v>497</v>
       </c>
-      <c r="B122" s="60" t="s">
-        <v>455</v>
-      </c>
-      <c r="C122" s="60" t="s">
+      <c r="D122" s="28" t="s">
         <v>498</v>
       </c>
-      <c r="D122" s="28" t="s">
+      <c r="E122" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F122" s="11" t="s">
         <v>499</v>
-      </c>
-      <c r="E122" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F122" s="11" t="s">
-        <v>500</v>
       </c>
       <c r="G122" s="11">
         <v>2</v>
       </c>
       <c r="H122" s="12" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
     </row>
     <row r="123" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A123" s="87" t="s">
+        <v>501</v>
+      </c>
+      <c r="B123" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="C123" s="60" t="s">
         <v>502</v>
       </c>
-      <c r="B123" s="60" t="s">
-        <v>455</v>
-      </c>
-      <c r="C123" s="60" t="s">
+      <c r="D123" s="28" t="s">
         <v>503</v>
       </c>
-      <c r="D123" s="28" t="s">
-        <v>504</v>
-      </c>
       <c r="E123" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F123" s="11" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="G123" s="11">
         <v>2</v>
       </c>
       <c r="H123" s="12" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="124" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A124" s="87" t="s">
+        <v>505</v>
+      </c>
+      <c r="B124" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="C124" s="60" t="s">
         <v>506</v>
       </c>
-      <c r="B124" s="60" t="s">
-        <v>455</v>
-      </c>
-      <c r="C124" s="60" t="s">
+      <c r="D124" s="28" t="s">
         <v>507</v>
       </c>
-      <c r="D124" s="28" t="s">
-        <v>508</v>
-      </c>
       <c r="E124" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F124" s="11" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="G124" s="11">
         <v>2</v>
       </c>
       <c r="H124" s="12" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A125" s="87" t="s">
+        <v>509</v>
+      </c>
+      <c r="B125" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="C125" s="60" t="s">
         <v>510</v>
       </c>
-      <c r="B125" s="60" t="s">
-        <v>455</v>
-      </c>
-      <c r="C125" s="60" t="s">
+      <c r="D125" s="28" t="s">
         <v>511</v>
       </c>
-      <c r="D125" s="28" t="s">
-        <v>512</v>
-      </c>
       <c r="E125" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F125" s="11" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="G125" s="11">
         <v>1</v>
       </c>
       <c r="H125" s="12" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A126" s="87" t="s">
+        <v>513</v>
+      </c>
+      <c r="B126" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="C126" s="60" t="s">
         <v>514</v>
       </c>
-      <c r="B126" s="60" t="s">
-        <v>455</v>
-      </c>
-      <c r="C126" s="60" t="s">
-        <v>515</v>
-      </c>
       <c r="D126" s="28" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="E126" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F126" s="11" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="G126" s="11">
         <v>2</v>
       </c>
       <c r="H126" s="12" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A127" s="87" t="s">
+        <v>516</v>
+      </c>
+      <c r="B127" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="C127" s="60" t="s">
         <v>517</v>
       </c>
-      <c r="B127" s="60" t="s">
-        <v>455</v>
-      </c>
-      <c r="C127" s="60" t="s">
+      <c r="D127" s="28" t="s">
         <v>518</v>
       </c>
-      <c r="D127" s="28" t="s">
-        <v>519</v>
-      </c>
       <c r="E127" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F127" s="11" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="G127" s="11">
         <v>3</v>
       </c>
       <c r="H127" s="12" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="128" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A128" s="87" t="s">
+        <v>520</v>
+      </c>
+      <c r="B128" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="C128" s="18" t="s">
         <v>521</v>
       </c>
-      <c r="B128" s="60" t="s">
-        <v>455</v>
-      </c>
-      <c r="C128" s="18" t="s">
+      <c r="D128" s="28" t="s">
         <v>522</v>
       </c>
-      <c r="D128" s="28" t="s">
-        <v>523</v>
-      </c>
       <c r="E128" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F128" s="11" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="G128" s="11">
         <v>4</v>
       </c>
       <c r="H128" s="12" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A129" s="87" t="s">
+        <v>524</v>
+      </c>
+      <c r="B129" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="C129" s="59" t="s">
         <v>525</v>
       </c>
-      <c r="B129" s="60" t="s">
-        <v>455</v>
-      </c>
-      <c r="C129" s="59" t="s">
+      <c r="D129" s="19" t="s">
         <v>526</v>
       </c>
-      <c r="D129" s="19" t="s">
-        <v>527</v>
-      </c>
       <c r="E129" s="2" t="s">
         <v>0</v>
       </c>
       <c r="F129" s="15" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="G129" s="15">
         <v>3</v>
       </c>
       <c r="H129" s="16" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
     </row>
     <row r="130" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A130" s="87" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B130" s="60" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C130" s="18" t="s">
         <v>42</v>
@@ -6046,42 +6047,42 @@
     </row>
     <row r="131" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A131" s="7" t="s">
+        <v>529</v>
+      </c>
+      <c r="B131" s="8" t="s">
         <v>530</v>
       </c>
-      <c r="B131" s="8" t="s">
+      <c r="C131" s="88" t="s">
         <v>531</v>
       </c>
-      <c r="C131" s="88" t="s">
+      <c r="D131" s="14" t="s">
         <v>532</v>
       </c>
-      <c r="D131" s="14" t="s">
+      <c r="E131" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F131" s="15" t="s">
         <v>533</v>
-      </c>
-      <c r="E131" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F131" s="15" t="s">
-        <v>534</v>
       </c>
       <c r="G131" s="15">
         <v>3</v>
       </c>
       <c r="H131" s="16" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
     </row>
     <row r="132" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A132" s="7" t="s">
+        <v>535</v>
+      </c>
+      <c r="B132" s="8" t="s">
+        <v>530</v>
+      </c>
+      <c r="C132" s="9" t="s">
         <v>536</v>
       </c>
-      <c r="B132" s="8" t="s">
-        <v>531</v>
-      </c>
-      <c r="C132" s="9" t="s">
+      <c r="D132" s="9" t="s">
         <v>537</v>
-      </c>
-      <c r="D132" s="9" t="s">
-        <v>538</v>
       </c>
       <c r="E132" s="10" t="s">
         <v>11</v>
@@ -6099,16 +6100,16 @@
     </row>
     <row r="133" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A133" s="7" t="s">
+        <v>538</v>
+      </c>
+      <c r="B133" s="8" t="s">
+        <v>530</v>
+      </c>
+      <c r="C133" s="9" t="s">
         <v>539</v>
       </c>
-      <c r="B133" s="8" t="s">
-        <v>531</v>
-      </c>
-      <c r="C133" s="9" t="s">
+      <c r="D133" s="9" t="s">
         <v>540</v>
-      </c>
-      <c r="D133" s="9" t="s">
-        <v>541</v>
       </c>
       <c r="E133" s="10" t="s">
         <v>11</v>
@@ -6123,88 +6124,88 @@
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A134" s="7" t="s">
+        <v>541</v>
+      </c>
+      <c r="B134" s="8" t="s">
+        <v>530</v>
+      </c>
+      <c r="C134" s="8" t="s">
         <v>542</v>
       </c>
-      <c r="B134" s="8" t="s">
-        <v>531</v>
-      </c>
-      <c r="C134" s="8" t="s">
+      <c r="D134" s="9" t="s">
         <v>543</v>
       </c>
-      <c r="D134" s="9" t="s">
+      <c r="E134" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F134" s="11" t="s">
         <v>544</v>
-      </c>
-      <c r="E134" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F134" s="11" t="s">
-        <v>545</v>
       </c>
       <c r="G134" s="11"/>
       <c r="H134" s="12" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A135" s="7" t="s">
+        <v>546</v>
+      </c>
+      <c r="B135" s="8" t="s">
+        <v>530</v>
+      </c>
+      <c r="C135" s="8" t="s">
         <v>547</v>
       </c>
-      <c r="B135" s="8" t="s">
-        <v>531</v>
-      </c>
-      <c r="C135" s="8" t="s">
+      <c r="D135" s="9" t="s">
         <v>548</v>
       </c>
-      <c r="D135" s="9" t="s">
-        <v>549</v>
-      </c>
       <c r="E135" s="10" t="s">
         <v>0</v>
       </c>
       <c r="F135" s="11" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="G135" s="11"/>
       <c r="H135" s="12" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
     </row>
     <row r="136" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A136" s="7" t="s">
+        <v>550</v>
+      </c>
+      <c r="B136" s="8" t="s">
+        <v>530</v>
+      </c>
+      <c r="C136" s="8" t="s">
         <v>551</v>
       </c>
-      <c r="B136" s="8" t="s">
-        <v>531</v>
-      </c>
-      <c r="C136" s="8" t="s">
+      <c r="D136" s="9" t="s">
         <v>552</v>
       </c>
-      <c r="D136" s="9" t="s">
+      <c r="E136" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F136" s="11" t="s">
         <v>553</v>
-      </c>
-      <c r="E136" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F136" s="11" t="s">
-        <v>554</v>
       </c>
       <c r="G136" s="11"/>
       <c r="H136" s="12" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
     </row>
     <row r="137" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A137" s="7" t="s">
+        <v>555</v>
+      </c>
+      <c r="B137" s="8" t="s">
+        <v>530</v>
+      </c>
+      <c r="C137" s="9" t="s">
         <v>556</v>
       </c>
-      <c r="B137" s="8" t="s">
-        <v>531</v>
-      </c>
-      <c r="C137" s="9" t="s">
+      <c r="D137" s="9" t="s">
         <v>557</v>
-      </c>
-      <c r="D137" s="9" t="s">
-        <v>558</v>
       </c>
       <c r="E137" s="10" t="s">
         <v>11</v>
@@ -6219,16 +6220,16 @@
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A138" s="7" t="s">
+        <v>558</v>
+      </c>
+      <c r="B138" s="8" t="s">
+        <v>530</v>
+      </c>
+      <c r="C138" s="48" t="s">
         <v>559</v>
       </c>
-      <c r="B138" s="8" t="s">
-        <v>531</v>
-      </c>
-      <c r="C138" s="48" t="s">
+      <c r="D138" s="9" t="s">
         <v>560</v>
-      </c>
-      <c r="D138" s="9" t="s">
-        <v>561</v>
       </c>
       <c r="E138" s="10" t="s">
         <v>11</v>
@@ -6243,26 +6244,26 @@
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A139" s="7" t="s">
+        <v>561</v>
+      </c>
+      <c r="B139" s="8" t="s">
+        <v>530</v>
+      </c>
+      <c r="C139" s="88" t="s">
         <v>562</v>
       </c>
-      <c r="B139" s="8" t="s">
-        <v>531</v>
-      </c>
-      <c r="C139" s="88" t="s">
+      <c r="D139" s="14" t="s">
         <v>563</v>
       </c>
-      <c r="D139" s="14" t="s">
+      <c r="E139" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F139" s="15" t="s">
         <v>564</v>
-      </c>
-      <c r="E139" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F139" s="15" t="s">
-        <v>565</v>
       </c>
       <c r="G139" s="15"/>
       <c r="H139" s="16" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="140" spans="1:8" x14ac:dyDescent="0.25">
@@ -6287,17 +6288,17 @@
     </row>
     <row r="143" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B143" s="6" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="144" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B144" s="6" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="145" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B145" s="6" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
   </sheetData>

</xml_diff>